<commit_message>
Use 15 percent lab detachment threshold
</commit_message>
<xml_diff>
--- a/outputs/lab_trials/lab_trials_repeatability_report.xlsx
+++ b/outputs/lab_trials/lab_trials_repeatability_report.xlsx
@@ -1514,7 +1514,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>A time is reported only if a positive change point reaches the pre-deposition minus 10% threshold. Otherwise the status is partial.</t>
+          <t>A time is reported only if a positive change point reaches the pre-deposition minus 15% threshold. Otherwise the status is partial.</t>
         </is>
       </c>
     </row>
@@ -9227,7 +9227,7 @@
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>threshold_10pct_lower</t>
+          <t>threshold_15pct_lower</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
@@ -9306,7 +9306,7 @@
         <v>0.5999351032931708</v>
       </c>
       <c r="M2" t="n">
-        <v>0.5399415929638537</v>
+        <v>0.5099448377991952</v>
       </c>
       <c r="N2" t="n">
         <v>0.7190809296697804</v>
@@ -9324,7 +9324,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 10%-below-pre-deposition-reference threshold</t>
+          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 15%-below-pre-deposition-reference threshold</t>
         </is>
       </c>
     </row>
@@ -9378,7 +9378,7 @@
         <v>0.6320859822554428</v>
       </c>
       <c r="M3" t="n">
-        <v>0.5688773840298985</v>
+        <v>0.5372730849171263</v>
       </c>
       <c r="N3" t="n">
         <v>0.5741389473170442</v>
@@ -9396,7 +9396,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 10%-below-pre-deposition-reference threshold</t>
+          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 15%-below-pre-deposition-reference threshold</t>
         </is>
       </c>
     </row>
@@ -9450,7 +9450,7 @@
         <v>0.5987148042124908</v>
       </c>
       <c r="M4" t="n">
-        <v>0.5388433237912417</v>
+        <v>0.5089075835806172</v>
       </c>
       <c r="N4" t="n">
         <v>0.700974947831748</v>
@@ -9468,7 +9468,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 10%-below-pre-deposition-reference threshold</t>
+          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 15%-below-pre-deposition-reference threshold</t>
         </is>
       </c>
     </row>
@@ -9511,7 +9511,7 @@
         <v>3140</v>
       </c>
       <c r="J5" t="n">
-        <v>2000.000344991684</v>
+        <v>1880.000734806061</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -9522,25 +9522,25 @@
         <v>0.6368147672906723</v>
       </c>
       <c r="M5" t="n">
-        <v>0.5731332905616051</v>
+        <v>0.5412925521970715</v>
       </c>
       <c r="N5" t="n">
-        <v>0.8339975784746477</v>
+        <v>0.5454090153670035</v>
       </c>
       <c r="O5" t="n">
         <v>3</v>
       </c>
       <c r="P5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>3 positive upward change points from detachment onset 1630.0s to cooling-window end 3140.0s. First passing point at 2000.0s.</t>
+          <t>3 positive upward change points from detachment onset 1630.0s to cooling-window end 3140.0s. First passing point at 1880.0s.</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 10%-below-pre-deposition-reference threshold</t>
+          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 15%-below-pre-deposition-reference threshold</t>
         </is>
       </c>
     </row>
@@ -9594,7 +9594,7 @@
         <v>0.6009845186289722</v>
       </c>
       <c r="M6" t="n">
-        <v>0.540886066766075</v>
+        <v>0.5108368408346263</v>
       </c>
       <c r="N6" t="n">
         <v>0.592980817588733</v>
@@ -9612,7 +9612,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 10%-below-pre-deposition-reference threshold</t>
+          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 15%-below-pre-deposition-reference threshold</t>
         </is>
       </c>
     </row>
@@ -9666,7 +9666,7 @@
         <v>0.6420872673309568</v>
       </c>
       <c r="M7" t="n">
-        <v>0.5778785405978611</v>
+        <v>0.5457741772313133</v>
       </c>
       <c r="N7" t="n">
         <v>0.8325951321135664</v>
@@ -9684,7 +9684,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 10%-below-pre-deposition-reference threshold</t>
+          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 15%-below-pre-deposition-reference threshold</t>
         </is>
       </c>
     </row>
@@ -9738,7 +9738,7 @@
         <v>0.7328215931830352</v>
       </c>
       <c r="M8" t="n">
-        <v>0.6595394338647317</v>
+        <v>0.6228983542055799</v>
       </c>
       <c r="N8" t="n">
         <v>0.821605322397148</v>
@@ -9756,7 +9756,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 10%-below-pre-deposition-reference threshold</t>
+          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 15%-below-pre-deposition-reference threshold</t>
         </is>
       </c>
     </row>
@@ -9798,16 +9798,19 @@
       <c r="I9" t="n">
         <v>2195</v>
       </c>
+      <c r="J9" t="n">
+        <v>1005.002333641052</v>
+      </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>partial_detachment_no_change_point_met_threshold</t>
+          <t>full_detachment_for_channel</t>
         </is>
       </c>
       <c r="L9" t="n">
         <v>0.6514162486792798</v>
       </c>
       <c r="M9" t="n">
-        <v>0.5862746238113519</v>
+        <v>0.5537038113773879</v>
       </c>
       <c r="N9" t="n">
         <v>0.5637620750490631</v>
@@ -9820,12 +9823,12 @@
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>4 positive upward change points from detachment onset 595.0s to cooling-window end 2195.0s. No change point reached the pre-deposition -10% threshold.</t>
+          <t>4 positive upward change points from detachment onset 595.0s to cooling-window end 2195.0s. First passing point at 1005.0s.</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 10%-below-pre-deposition-reference threshold</t>
+          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 15%-below-pre-deposition-reference threshold</t>
         </is>
       </c>
     </row>
@@ -9879,7 +9882,7 @@
         <v>0.7407382036638537</v>
       </c>
       <c r="M10" t="n">
-        <v>0.6666643832974684</v>
+        <v>0.6296274731142756</v>
       </c>
       <c r="N10" t="n">
         <v>0.9000121704076206</v>
@@ -9897,7 +9900,7 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 10%-below-pre-deposition-reference threshold</t>
+          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 15%-below-pre-deposition-reference threshold</t>
         </is>
       </c>
     </row>
@@ -9951,7 +9954,7 @@
         <v>0.6669369645234606</v>
       </c>
       <c r="M11" t="n">
-        <v>0.6002432680711146</v>
+        <v>0.5668964198449415</v>
       </c>
       <c r="N11" t="n">
         <v>0.699081120081692</v>
@@ -9969,7 +9972,7 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 10%-below-pre-deposition-reference threshold</t>
+          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 15%-below-pre-deposition-reference threshold</t>
         </is>
       </c>
     </row>
@@ -10023,7 +10026,7 @@
         <v>0.7293372337684932</v>
       </c>
       <c r="M12" t="n">
-        <v>0.6564035103916439</v>
+        <v>0.6199366487032193</v>
       </c>
       <c r="N12" t="n">
         <v>0.856245613560319</v>
@@ -10041,7 +10044,7 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 10%-below-pre-deposition-reference threshold</t>
+          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 15%-below-pre-deposition-reference threshold</t>
         </is>
       </c>
     </row>
@@ -10092,7 +10095,7 @@
         <v>0.6557684022430149</v>
       </c>
       <c r="M13" t="n">
-        <v>0.5901915620187135</v>
+        <v>0.5574031419065627</v>
       </c>
       <c r="N13" t="n">
         <v>0.485939799054226</v>
@@ -10105,12 +10108,12 @@
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>3 positive upward change points from detachment onset 1064.0s to cooling-window end 2694.0s. No change point reached the pre-deposition -10% threshold.</t>
+          <t>3 positive upward change points from detachment onset 1064.0s to cooling-window end 2694.0s. No change point reached the pre-deposition -15% threshold.</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 10%-below-pre-deposition-reference threshold</t>
+          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 15%-below-pre-deposition-reference threshold</t>
         </is>
       </c>
     </row>
@@ -10161,7 +10164,7 @@
         <v>0.5923920642654367</v>
       </c>
       <c r="M14" t="n">
-        <v>0.533152857838893</v>
+        <v>0.5035332546256212</v>
       </c>
       <c r="N14" t="n">
         <v>0.2876314729136664</v>
@@ -10174,12 +10177,12 @@
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>2 positive upward change points from detachment onset 1094.0s to cooling-window end 2261.0s. No change point reached the pre-deposition -10% threshold.</t>
+          <t>2 positive upward change points from detachment onset 1094.0s to cooling-window end 2261.0s. No change point reached the pre-deposition -15% threshold.</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 10%-below-pre-deposition-reference threshold</t>
+          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 15%-below-pre-deposition-reference threshold</t>
         </is>
       </c>
     </row>
@@ -10233,7 +10236,7 @@
         <v>0.5936340750157071</v>
       </c>
       <c r="M15" t="n">
-        <v>0.5342706675141364</v>
+        <v>0.5045889637633511</v>
       </c>
       <c r="N15" t="n">
         <v>0.6549491860507034</v>
@@ -10251,7 +10254,7 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 10%-below-pre-deposition-reference threshold</t>
+          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 15%-below-pre-deposition-reference threshold</t>
         </is>
       </c>
     </row>
@@ -10302,7 +10305,7 @@
         <v>0.5855064536151028</v>
       </c>
       <c r="M16" t="n">
-        <v>0.5269558082535926</v>
+        <v>0.4976804855728374</v>
       </c>
       <c r="N16" t="n">
         <v>0.4375577006045251</v>
@@ -10315,12 +10318,12 @@
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>3 positive upward change points from detachment onset 783.0s to cooling-window end 2072.0s. No change point reached the pre-deposition -10% threshold.</t>
+          <t>3 positive upward change points from detachment onset 783.0s to cooling-window end 2072.0s. No change point reached the pre-deposition -15% threshold.</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 10%-below-pre-deposition-reference threshold</t>
+          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 15%-below-pre-deposition-reference threshold</t>
         </is>
       </c>
     </row>
@@ -10374,7 +10377,7 @@
         <v>0.6034922114924255</v>
       </c>
       <c r="M17" t="n">
-        <v>0.5431429903431829</v>
+        <v>0.5129683797685617</v>
       </c>
       <c r="N17" t="n">
         <v>0.7775187872829324</v>
@@ -10392,7 +10395,7 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 10%-below-pre-deposition-reference threshold</t>
+          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 15%-below-pre-deposition-reference threshold</t>
         </is>
       </c>
     </row>
@@ -10434,16 +10437,19 @@
       <c r="I18" t="n">
         <v>2017</v>
       </c>
+      <c r="J18" t="n">
+        <v>1413.9799451828</v>
+      </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>partial_detachment_no_change_point_met_threshold</t>
+          <t>full_detachment_for_channel</t>
         </is>
       </c>
       <c r="L18" t="n">
         <v>0.6090918111618937</v>
       </c>
       <c r="M18" t="n">
-        <v>0.5481826300457043</v>
+        <v>0.5177280394876096</v>
       </c>
       <c r="N18" t="n">
         <v>0.5421488160143766</v>
@@ -10456,12 +10462,12 @@
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>2 positive upward change points from detachment onset 1000.0s to cooling-window end 2017.0s. No change point reached the pre-deposition -10% threshold.</t>
+          <t>2 positive upward change points from detachment onset 1000.0s to cooling-window end 2017.0s. First passing point at 1414.0s.</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 10%-below-pre-deposition-reference threshold</t>
+          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 15%-below-pre-deposition-reference threshold</t>
         </is>
       </c>
     </row>
@@ -10515,7 +10521,7 @@
         <v>0.6091249232898795</v>
       </c>
       <c r="M19" t="n">
-        <v>0.5482124309608916</v>
+        <v>0.5177561847963976</v>
       </c>
       <c r="N19" t="n">
         <v>0.7454181265800934</v>
@@ -10533,7 +10539,7 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 10%-below-pre-deposition-reference threshold</t>
+          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 15%-below-pre-deposition-reference threshold</t>
         </is>
       </c>
     </row>
@@ -10587,7 +10593,7 @@
         <v>0.6207563871985903</v>
       </c>
       <c r="M20" t="n">
-        <v>0.5586807484787313</v>
+        <v>0.5276429291188017</v>
       </c>
       <c r="N20" t="n">
         <v>0.6579884605851972</v>
@@ -10605,7 +10611,7 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 10%-below-pre-deposition-reference threshold</t>
+          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 15%-below-pre-deposition-reference threshold</t>
         </is>
       </c>
     </row>
@@ -10659,7 +10665,7 @@
         <v>0.609385090085468</v>
       </c>
       <c r="M21" t="n">
-        <v>0.5484465810769212</v>
+        <v>0.5179773265726478</v>
       </c>
       <c r="N21" t="n">
         <v>0.8044727888986035</v>
@@ -10677,7 +10683,7 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 10%-below-pre-deposition-reference threshold</t>
+          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 15%-below-pre-deposition-reference threshold</t>
         </is>
       </c>
     </row>
@@ -10728,7 +10734,7 @@
         <v>0.6199542903035502</v>
       </c>
       <c r="M22" t="n">
-        <v>0.5579588612731952</v>
+        <v>0.5269611467580176</v>
       </c>
       <c r="N22" t="n">
         <v>0.4578294486704634</v>
@@ -10741,12 +10747,12 @@
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>5 positive upward change points from detachment onset 1228.0s to cooling-window end 2515.0s. No change point reached the pre-deposition -10% threshold.</t>
+          <t>5 positive upward change points from detachment onset 1228.0s to cooling-window end 2515.0s. No change point reached the pre-deposition -15% threshold.</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 10%-below-pre-deposition-reference threshold</t>
+          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 15%-below-pre-deposition-reference threshold</t>
         </is>
       </c>
     </row>
@@ -10800,7 +10806,7 @@
         <v>0.6023667048574612</v>
       </c>
       <c r="M23" t="n">
-        <v>0.5421300343717151</v>
+        <v>0.512011699128842</v>
       </c>
       <c r="N23" t="n">
         <v>0.7621613005628776</v>
@@ -10818,7 +10824,7 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 10%-below-pre-deposition-reference threshold</t>
+          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 15%-below-pre-deposition-reference threshold</t>
         </is>
       </c>
     </row>
@@ -10869,7 +10875,7 @@
         <v>0.6274948017835749</v>
       </c>
       <c r="M24" t="n">
-        <v>0.5647453216052174</v>
+        <v>0.5333705815160387</v>
       </c>
       <c r="N24" t="n">
         <v>0.4457565432800725</v>
@@ -10882,12 +10888,12 @@
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>3 positive upward change points from detachment onset 1217.0s to cooling-window end 2500.0s. No change point reached the pre-deposition -10% threshold.</t>
+          <t>3 positive upward change points from detachment onset 1217.0s to cooling-window end 2500.0s. No change point reached the pre-deposition -15% threshold.</t>
         </is>
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 10%-below-pre-deposition-reference threshold</t>
+          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 15%-below-pre-deposition-reference threshold</t>
         </is>
       </c>
     </row>
@@ -10941,7 +10947,7 @@
         <v>0.6077120963216972</v>
       </c>
       <c r="M25" t="n">
-        <v>0.5469408866895275</v>
+        <v>0.5165552818734427</v>
       </c>
       <c r="N25" t="n">
         <v>0.7769129392553277</v>
@@ -10959,7 +10965,7 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 10%-below-pre-deposition-reference threshold</t>
+          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 15%-below-pre-deposition-reference threshold</t>
         </is>
       </c>
     </row>
@@ -11044,7 +11050,7 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>threshold_10pct_lower</t>
+          <t>threshold_15pct_lower</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
@@ -11117,7 +11123,7 @@
         <v>0.5999351032931708</v>
       </c>
       <c r="J2" t="n">
-        <v>0.5399415929638537</v>
+        <v>0.5099448377991952</v>
       </c>
       <c r="K2" t="n">
         <v>0.7190809296697804</v>
@@ -11183,7 +11189,7 @@
         <v>0.6320859822554428</v>
       </c>
       <c r="J3" t="n">
-        <v>0.5688773840298985</v>
+        <v>0.5372730849171263</v>
       </c>
       <c r="K3" t="n">
         <v>0.5741389473170442</v>
@@ -11249,7 +11255,7 @@
         <v>0.5987148042124908</v>
       </c>
       <c r="J4" t="n">
-        <v>0.5388433237912417</v>
+        <v>0.5089075835806172</v>
       </c>
       <c r="K4" t="n">
         <v>0.700974947831748</v>
@@ -11309,26 +11315,26 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>2000.000344991684</v>
+        <v>1880.000734806061</v>
       </c>
       <c r="I5" t="n">
         <v>0.6368147672906723</v>
       </c>
       <c r="J5" t="n">
-        <v>0.5731332905616051</v>
+        <v>0.5412925521970715</v>
       </c>
       <c r="K5" t="n">
-        <v>0.8339975784746477</v>
+        <v>0.5454090153670035</v>
       </c>
       <c r="L5" t="n">
         <v>3</v>
       </c>
       <c r="M5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>3 positive upward change points from detachment onset 1630.0s to cooling-window end 3140.0s. First passing point at 2000.0s.</t>
+          <t>3 positive upward change points from detachment onset 1630.0s to cooling-window end 3140.0s. First passing point at 1880.0s.</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -11338,7 +11344,7 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>2 change points before full detachment offset</t>
+          <t>1 change points before full detachment offset</t>
         </is>
       </c>
     </row>
@@ -11381,7 +11387,7 @@
         <v>0.6009845186289722</v>
       </c>
       <c r="J6" t="n">
-        <v>0.540886066766075</v>
+        <v>0.5108368408346263</v>
       </c>
       <c r="K6" t="n">
         <v>0.592980817588733</v>
@@ -11447,7 +11453,7 @@
         <v>0.6420872673309568</v>
       </c>
       <c r="J7" t="n">
-        <v>0.5778785405978611</v>
+        <v>0.5457741772313133</v>
       </c>
       <c r="K7" t="n">
         <v>0.8325951321135664</v>
@@ -11513,7 +11519,7 @@
         <v>0.7328215931830352</v>
       </c>
       <c r="J8" t="n">
-        <v>0.6595394338647317</v>
+        <v>0.6228983542055799</v>
       </c>
       <c r="K8" t="n">
         <v>0.821605322397148</v>
@@ -11569,14 +11575,17 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>partial_detachment_no_change_point_met_threshold</t>
-        </is>
+          <t>full_detachment_for_channel</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>1005.002333641052</v>
       </c>
       <c r="I9" t="n">
         <v>0.6514162486792798</v>
       </c>
       <c r="J9" t="n">
-        <v>0.5862746238113519</v>
+        <v>0.5537038113773879</v>
       </c>
       <c r="K9" t="n">
         <v>0.5637620750490631</v>
@@ -11589,7 +11598,7 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>4 positive upward change points from detachment onset 595.0s to cooling-window end 2195.0s. No change point reached the pre-deposition -10% threshold.</t>
+          <t>4 positive upward change points from detachment onset 595.0s to cooling-window end 2195.0s. First passing point at 1005.0s.</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
@@ -11599,7 +11608,7 @@
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>4 change points checked; no full detachment offset</t>
+          <t>4 change points before full detachment offset</t>
         </is>
       </c>
     </row>
@@ -11642,7 +11651,7 @@
         <v>0.7407382036638537</v>
       </c>
       <c r="J10" t="n">
-        <v>0.6666643832974684</v>
+        <v>0.6296274731142756</v>
       </c>
       <c r="K10" t="n">
         <v>0.9000121704076206</v>
@@ -11708,7 +11717,7 @@
         <v>0.6669369645234606</v>
       </c>
       <c r="J11" t="n">
-        <v>0.6002432680711146</v>
+        <v>0.5668964198449415</v>
       </c>
       <c r="K11" t="n">
         <v>0.699081120081692</v>
@@ -11774,7 +11783,7 @@
         <v>0.7293372337684932</v>
       </c>
       <c r="J12" t="n">
-        <v>0.6564035103916439</v>
+        <v>0.6199366487032193</v>
       </c>
       <c r="K12" t="n">
         <v>0.856245613560319</v>
@@ -11837,7 +11846,7 @@
         <v>0.6557684022430149</v>
       </c>
       <c r="J13" t="n">
-        <v>0.5901915620187135</v>
+        <v>0.5574031419065627</v>
       </c>
       <c r="K13" t="n">
         <v>0.485939799054226</v>
@@ -11850,7 +11859,7 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>3 positive upward change points from detachment onset 1064.0s to cooling-window end 2694.0s. No change point reached the pre-deposition -10% threshold.</t>
+          <t>3 positive upward change points from detachment onset 1064.0s to cooling-window end 2694.0s. No change point reached the pre-deposition -15% threshold.</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
@@ -11900,7 +11909,7 @@
         <v>0.5923920642654367</v>
       </c>
       <c r="J14" t="n">
-        <v>0.533152857838893</v>
+        <v>0.5035332546256212</v>
       </c>
       <c r="K14" t="n">
         <v>0.2876314729136664</v>
@@ -11913,7 +11922,7 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>2 positive upward change points from detachment onset 1094.0s to cooling-window end 2261.0s. No change point reached the pre-deposition -10% threshold.</t>
+          <t>2 positive upward change points from detachment onset 1094.0s to cooling-window end 2261.0s. No change point reached the pre-deposition -15% threshold.</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
@@ -11966,7 +11975,7 @@
         <v>0.5936340750157071</v>
       </c>
       <c r="J15" t="n">
-        <v>0.5342706675141364</v>
+        <v>0.5045889637633511</v>
       </c>
       <c r="K15" t="n">
         <v>0.6549491860507034</v>
@@ -12029,7 +12038,7 @@
         <v>0.5855064536151028</v>
       </c>
       <c r="J16" t="n">
-        <v>0.5269558082535926</v>
+        <v>0.4976804855728374</v>
       </c>
       <c r="K16" t="n">
         <v>0.4375577006045251</v>
@@ -12042,7 +12051,7 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>3 positive upward change points from detachment onset 783.0s to cooling-window end 2072.0s. No change point reached the pre-deposition -10% threshold.</t>
+          <t>3 positive upward change points from detachment onset 783.0s to cooling-window end 2072.0s. No change point reached the pre-deposition -15% threshold.</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
@@ -12095,7 +12104,7 @@
         <v>0.6034922114924255</v>
       </c>
       <c r="J17" t="n">
-        <v>0.5431429903431829</v>
+        <v>0.5129683797685617</v>
       </c>
       <c r="K17" t="n">
         <v>0.7775187872829324</v>
@@ -12151,14 +12160,17 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>partial_detachment_no_change_point_met_threshold</t>
-        </is>
+          <t>full_detachment_for_channel</t>
+        </is>
+      </c>
+      <c r="H18" t="n">
+        <v>1413.9799451828</v>
       </c>
       <c r="I18" t="n">
         <v>0.6090918111618937</v>
       </c>
       <c r="J18" t="n">
-        <v>0.5481826300457043</v>
+        <v>0.5177280394876096</v>
       </c>
       <c r="K18" t="n">
         <v>0.5421488160143766</v>
@@ -12171,7 +12183,7 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>2 positive upward change points from detachment onset 1000.0s to cooling-window end 2017.0s. No change point reached the pre-deposition -10% threshold.</t>
+          <t>2 positive upward change points from detachment onset 1000.0s to cooling-window end 2017.0s. First passing point at 1414.0s.</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
@@ -12181,7 +12193,7 @@
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>2 change points checked; no full detachment offset</t>
+          <t>2 change points before full detachment offset</t>
         </is>
       </c>
     </row>
@@ -12224,7 +12236,7 @@
         <v>0.6091249232898795</v>
       </c>
       <c r="J19" t="n">
-        <v>0.5482124309608916</v>
+        <v>0.5177561847963976</v>
       </c>
       <c r="K19" t="n">
         <v>0.7454181265800934</v>
@@ -12290,7 +12302,7 @@
         <v>0.6207563871985903</v>
       </c>
       <c r="J20" t="n">
-        <v>0.5586807484787313</v>
+        <v>0.5276429291188017</v>
       </c>
       <c r="K20" t="n">
         <v>0.6579884605851972</v>
@@ -12356,7 +12368,7 @@
         <v>0.609385090085468</v>
       </c>
       <c r="J21" t="n">
-        <v>0.5484465810769212</v>
+        <v>0.5179773265726478</v>
       </c>
       <c r="K21" t="n">
         <v>0.8044727888986035</v>
@@ -12419,7 +12431,7 @@
         <v>0.6199542903035502</v>
       </c>
       <c r="J22" t="n">
-        <v>0.5579588612731952</v>
+        <v>0.5269611467580176</v>
       </c>
       <c r="K22" t="n">
         <v>0.4578294486704634</v>
@@ -12432,7 +12444,7 @@
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>5 positive upward change points from detachment onset 1228.0s to cooling-window end 2515.0s. No change point reached the pre-deposition -10% threshold.</t>
+          <t>5 positive upward change points from detachment onset 1228.0s to cooling-window end 2515.0s. No change point reached the pre-deposition -15% threshold.</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
@@ -12485,7 +12497,7 @@
         <v>0.6023667048574612</v>
       </c>
       <c r="J23" t="n">
-        <v>0.5421300343717151</v>
+        <v>0.512011699128842</v>
       </c>
       <c r="K23" t="n">
         <v>0.7621613005628776</v>
@@ -12548,7 +12560,7 @@
         <v>0.6274948017835749</v>
       </c>
       <c r="J24" t="n">
-        <v>0.5647453216052174</v>
+        <v>0.5333705815160387</v>
       </c>
       <c r="K24" t="n">
         <v>0.4457565432800725</v>
@@ -12561,7 +12573,7 @@
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>3 positive upward change points from detachment onset 1217.0s to cooling-window end 2500.0s. No change point reached the pre-deposition -10% threshold.</t>
+          <t>3 positive upward change points from detachment onset 1217.0s to cooling-window end 2500.0s. No change point reached the pre-deposition -15% threshold.</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
@@ -12614,7 +12626,7 @@
         <v>0.6077120963216972</v>
       </c>
       <c r="J25" t="n">
-        <v>0.5469408866895275</v>
+        <v>0.5165552818734427</v>
       </c>
       <c r="K25" t="n">
         <v>0.7769129392553277</v>

</xml_diff>

<commit_message>
Add detachment CV and comparison figures
</commit_message>
<xml_diff>
--- a/outputs/lab_trials/lab_trials_repeatability_report.xlsx
+++ b/outputs/lab_trials/lab_trials_repeatability_report.xlsx
@@ -11,22 +11,25 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1 Summary Factor Effects" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2 Repeatability CV" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3 Temp Explains Outcomes" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4 Detachment Summary vs US" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5 Detachment Statistics" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="US Rupture Decisions" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="US Change Points" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zone and US Figures" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rupture Decision Figures" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4 Detachment CV" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5 Detachment Summary vs US" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6 Detachment Statistics" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="US Rupture Decisions" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="US Change Points" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detachment Comparison Figures" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zone and US Figures" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rupture Decision Figures" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Read Me'!$A$1:$D$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Read Me'!$A$1:$D$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'1 Summary Factor Effects'!$A$1:$H$50</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'2 Repeatability CV'!$A$1:$L$57</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'3 Temp Explains Outcomes'!$A$1:$N$41</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'4 Detachment Summary vs US'!$A$1:$AB$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'5 Detachment Statistics'!$A$1:$K$89</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'US Rupture Decisions'!$A$1:$R$25</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'US Change Points'!$A$1:$P$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'4 Detachment CV'!$A$1:$L$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'5 Detachment Summary vs US'!$A$1:$AB$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'6 Detachment Statistics'!$A$1:$K$89</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'US Rupture Decisions'!$A$1:$R$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'US Change Points'!$A$1:$P$25</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -155,6 +158,86 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="9334500" cy="5276850"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>35</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="9334500" cy="5276850"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId2"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>69</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="9334500" cy="5276850"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId3"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -509,7 +592,7 @@
 </wsDr>
 </file>
 
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -1403,7 +1486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1508,17 +1591,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>4 Detachment Summary vs US</t>
+          <t>4 Detachment CV</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Do manually summarized detachment completion/duration and US-derived detachment offset agree?</t>
+          <t>How repeatable are detachment duration, offset differences, and change-point counts within each experiment set?</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Rx2Tx2 is used as the preferred channel when present. Rx1Tx1 and Rx2Tx2 are both kept in separate columns so channel disagreement is visible.</t>
+          <t>This is the preliminary within-set CV check. A high Trials effect later means sets differ from each other; high CV here means repetitions inside the same set are not repeatable.</t>
         </is>
       </c>
     </row>
@@ -1530,17 +1613,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>5 Detachment Statistics</t>
+          <t>5 Detachment Summary vs US</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Which experimental factors are associated with detachment duration, full-offset probability, and change-point count?</t>
+          <t>Do manually summarized detachment completion/duration and US-derived detachment offset agree?</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Eta-squared screens setup effects; correlation rows compare summary-derived and US-derived detachment behavior. Treat this as exploratory because n is small.</t>
+          <t>Rx2Tx2 is used as the preferred channel when present. Rx1Tx1 and Rx2Tx2 are both kept in separate columns so channel disagreement is visible.</t>
         </is>
       </c>
     </row>
@@ -1552,17 +1635,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>US Rupture Decisions</t>
+          <t>6 Detachment Statistics</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>For each repetition, sensor code, and primary US channel, was full detachment reached and at what offset time?</t>
+          <t>Which experimental factors are associated with detachment duration, full-offset probability, and change-point count?</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>A time is reported only if a positive change point reaches the pre-deposition minus 15% threshold. Otherwise the status is partial.</t>
+          <t>Eta-squared screens setup effects; correlation rows compare summary-derived and US-derived detachment behavior. Treat this as exploratory because n is small.</t>
         </is>
       </c>
     </row>
@@ -1574,17 +1657,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>US Change Points</t>
+          <t>US Rupture Decisions</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Which positive/upward US change points were detected and did they pass the threshold?</t>
+          <t>For each repetition, sensor code, and primary US channel, was full detachment reached and at what offset time?</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>This is the audit trail behind the detachment offset decision.</t>
+          <t>A time is reported only if a positive change point reaches the pre-deposition minus 15% threshold. Otherwise the status is partial.</t>
         </is>
       </c>
     </row>
@@ -1596,93 +1679,264 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Zone and US Figures / Rupture Decision Figures</t>
+          <t>US Change Points</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Visual checks for zones, onset, full-detachment offsets, rupture points, and threshold criteria.</t>
+          <t>Which positive/upward US change points were detected and did they pass the threshold?</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Red offset lines are only drawn where full detachment was detected.</t>
+          <t>This is the audit trail behind the detachment offset decision.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Zone note</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Zone and US Figures</t>
+          <t>Zone and US Figures / Rupture Decision Figures</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>How lab-device cooling zones are split.</t>
+          <t>Visual checks for zones, onset, full-detachment offsets, rupture points, and threshold criteria.</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>For non-test lab-device runs, Z2 is cooling simulator until the first rise pattern, Z3 is intermediate cooling simulator until the later strong warming/demoulding transition. a5 anchors this at about 2000 s and 2550 s.</t>
+          <t>Red offset lines are only drawn where full detachment was detected.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Caution</t>
+          <t>Zone note</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>All sheets</t>
+          <t>Zone and US Figures</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Statistical meaning</t>
+          <t>How lab-device cooling zones are split.</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>These are exploratory effect sizes and correlations. With few repetitions, they are pattern evidence and prioritization, not formal proof.</t>
+          <t>For non-test lab-device runs, Z2 is cooling simulator until the first rise pattern, Z3 is intermediate cooling simulator until the later strong warming/demoulding transition. a5 anchors this at about 2000 s and 2550 s.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>Caution</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>All sheets</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Statistical meaning</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>These are exploratory effect sizes and correlations. With few repetitions, they are pattern evidence and prioritization, not formal proof.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t>Raw</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>inputs/lab_trials</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>Which raw workbook was rebuilt from the replacement CSV files?</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>C:\Users\BurkardJohannes\Documents\CHoNova _ Data Understanding\inputs\lab_trials\lab_trials_raw.xlsx</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D12"/>
+  <autoFilter ref="A1:D13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A69"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>detachment_duration_grouped_bars.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>detachment_change_point_counts_grouped_bars.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>detachment_offsets_grouped_bars.png</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A456"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>2455_a_test_zones_us_offsets.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2455_a_test3_zones_us_offsets.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2455_a_test4_zones_us_offsets.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>2455_a5_zones_us_offsets.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>2455_a6_zones_us_offsets.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>2455_a7_zones_us_offsets.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>2455_b_zones_us_offsets.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>2455_b2_zones_us_offsets.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>2455_b3_zones_us_offsets.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>2455_b4_zones_us_offsets.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>2561_a1_zones_us_offsets.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>2561_a2_zones_us_offsets.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>2561_a3_zones_us_offsets.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" t="inlineStr">
+        <is>
+          <t>2561_a4_zones_us_offsets.png</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -9372,6 +9626,1609 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:L31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="21" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="29" customWidth="1" min="11" max="11"/>
+    <col width="32" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>channel_or_scope</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>metric</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>metric_column</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>n_repetitions</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>std</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>cv_percent</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>min</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>max</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>repeatability_flag</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>interpretation</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2455_a5/a6/a7</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Rx1Tx1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Rx1Tx1 change-point count</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>rx1_change_points_until_offset_or_last</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>3</v>
+      </c>
+      <c r="F2" t="n">
+        <v>2.666666666666667</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.5773502691896258</v>
+      </c>
+      <c r="H2" t="n">
+        <v>21.65063509461097</v>
+      </c>
+      <c r="I2" t="n">
+        <v>2</v>
+      </c>
+      <c r="J2" t="n">
+        <v>3</v>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>low repeatability / inspect</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>2455_a5/a6/a7 Rx1Tx1 change-point count: CV 21.7%; low repeatability / inspect.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2455_a5/a6/a7</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Rx1Tx1</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Rx1Tx1 duration</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>rx1_detachment_duration_s</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F3" t="n">
+        <v>561.6681698958079</v>
+      </c>
+      <c r="G3" t="n">
+        <v>80.98296099587238</v>
+      </c>
+      <c r="H3" t="n">
+        <v>14.41829274585653</v>
+      </c>
+      <c r="I3" t="n">
+        <v>510.0024194717407</v>
+      </c>
+      <c r="J3" t="n">
+        <v>655.0008795261383</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>moderate repeatability</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2455_a5/a6/a7 Rx1Tx1 duration: CV 14.4%; moderate repeatability.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2455_a5/a6/a7</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Rx2Tx2</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Rx2Tx2 change-point count</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>rx2_change_points_until_offset_or_last</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>3</v>
+      </c>
+      <c r="F4" t="n">
+        <v>1.666666666666667</v>
+      </c>
+      <c r="G4" t="n">
+        <v>1.154700538379252</v>
+      </c>
+      <c r="H4" t="n">
+        <v>69.2820323027551</v>
+      </c>
+      <c r="I4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J4" t="n">
+        <v>3</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>low repeatability / inspect</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2455_a5/a6/a7 Rx2Tx2 change-point count: CV 69.3%; low repeatability / inspect.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2455_a5/a6/a7</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Rx2Tx2</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Rx2Tx2 duration</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>rx2_detachment_duration_s</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F5" t="n">
+        <v>269.9999094804127</v>
+      </c>
+      <c r="G5" t="n">
+        <v>62.45066399874025</v>
+      </c>
+      <c r="H5" t="n">
+        <v>23.12988330956117</v>
+      </c>
+      <c r="I5" t="n">
+        <v>219.9985785484312</v>
+      </c>
+      <c r="J5" t="n">
+        <v>340.0004150867462</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>low repeatability / inspect</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2455_a5/a6/a7 Rx2Tx2 duration: CV 23.1%; low repeatability / inspect.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2455_a5/a6/a7</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>channel_difference</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Rx2Tx2 minus Rx1Tx1 offset</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>rx2_minus_rx1_offset_s</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>3</v>
+      </c>
+      <c r="F6" t="n">
+        <v>-423.3349270820618</v>
+      </c>
+      <c r="G6" t="n">
+        <v>123.9279600163208</v>
+      </c>
+      <c r="H6" t="n">
+        <v>29.27421105329629</v>
+      </c>
+      <c r="I6" t="n">
+        <v>-535.0001447200775</v>
+      </c>
+      <c r="J6" t="n">
+        <v>-290.0020043849945</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>low repeatability / inspect</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2455_a5/a6/a7 Rx2Tx2 minus Rx1Tx1 offset: CV 29.3%; low repeatability / inspect.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2455_a5/a6/a7</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>preferred_us</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>preferred US change-point count</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>us_change_points_until_offset_or_last</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>3</v>
+      </c>
+      <c r="F7" t="n">
+        <v>1.666666666666667</v>
+      </c>
+      <c r="G7" t="n">
+        <v>1.154700538379252</v>
+      </c>
+      <c r="H7" t="n">
+        <v>69.2820323027551</v>
+      </c>
+      <c r="I7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J7" t="n">
+        <v>3</v>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>low repeatability / inspect</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2455_a5/a6/a7 preferred US change-point count: CV 69.3%; low repeatability / inspect.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2455_a5/a6/a7</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>preferred_us</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>preferred US duration</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>us_detachment_duration_s</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>3</v>
+      </c>
+      <c r="F8" t="n">
+        <v>269.9999094804127</v>
+      </c>
+      <c r="G8" t="n">
+        <v>62.45066399874025</v>
+      </c>
+      <c r="H8" t="n">
+        <v>23.12988330956117</v>
+      </c>
+      <c r="I8" t="n">
+        <v>219.9985785484312</v>
+      </c>
+      <c r="J8" t="n">
+        <v>340.0004150867462</v>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>low repeatability / inspect</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>2455_a5/a6/a7 preferred US duration: CV 23.1%; low repeatability / inspect.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2455_a5/a6/a7</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>summary duration</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>summary_detachment_duration_s</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>3</v>
+      </c>
+      <c r="F9" t="n">
+        <v>348.3333333333333</v>
+      </c>
+      <c r="G9" t="n">
+        <v>48.04511768466525</v>
+      </c>
+      <c r="H9" t="n">
+        <v>13.79285675157854</v>
+      </c>
+      <c r="I9" t="n">
+        <v>305</v>
+      </c>
+      <c r="J9" t="n">
+        <v>400</v>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>moderate repeatability</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>2455_a5/a6/a7 summary duration: CV 13.8%; moderate repeatability.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2455_a_test/test3/test4</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Rx1Tx1</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Rx1Tx1 change-point count</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>rx1_change_points_until_offset_or_last</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>3</v>
+      </c>
+      <c r="F10" t="n">
+        <v>2</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" t="n">
+        <v>2</v>
+      </c>
+      <c r="J10" t="n">
+        <v>2</v>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>high repeatability</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>2455_a_test/test3/test4 Rx1Tx1 change-point count: CV 0.0%; high repeatability.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2455_a_test/test3/test4</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Rx1Tx1</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Rx1Tx1 duration</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>rx1_detachment_duration_s</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>3</v>
+      </c>
+      <c r="F11" t="n">
+        <v>229.3341773351032</v>
+      </c>
+      <c r="G11" t="n">
+        <v>35.34705172763976</v>
+      </c>
+      <c r="H11" t="n">
+        <v>15.41290187898624</v>
+      </c>
+      <c r="I11" t="n">
+        <v>206.0005948543549</v>
+      </c>
+      <c r="J11" t="n">
+        <v>270.0022101402282</v>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>inspect</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>2455_a_test/test3/test4 Rx1Tx1 duration: CV 15.4%; inspect.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2455_a_test/test3/test4</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Rx2Tx2</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Rx2Tx2 change-point count</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>rx2_change_points_until_offset_or_last</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>3</v>
+      </c>
+      <c r="F12" t="n">
+        <v>3.666666666666667</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0.5773502691896258</v>
+      </c>
+      <c r="H12" t="n">
+        <v>15.74591643244434</v>
+      </c>
+      <c r="I12" t="n">
+        <v>3</v>
+      </c>
+      <c r="J12" t="n">
+        <v>4</v>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>inspect</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>2455_a_test/test3/test4 Rx2Tx2 change-point count: CV 15.7%; inspect.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2455_a_test/test3/test4</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Rx2Tx2</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Rx2Tx2 duration</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>rx2_detachment_duration_s</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>2</v>
+      </c>
+      <c r="F13" t="n">
+        <v>462.0011442899703</v>
+      </c>
+      <c r="G13" t="n">
+        <v>73.53742324697041</v>
+      </c>
+      <c r="H13" t="n">
+        <v>15.91715175510808</v>
+      </c>
+      <c r="I13" t="n">
+        <v>410.0023336410522</v>
+      </c>
+      <c r="J13" t="n">
+        <v>513.9999549388883</v>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>inspect</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>2455_a_test/test3/test4 Rx2Tx2 duration: CV 15.9%; inspect.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2455_a_test/test3/test4</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>channel_difference</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Rx2Tx2 minus Rx1Tx1 offset</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>rx2_minus_rx1_offset_s</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>2</v>
+      </c>
+      <c r="F14" t="n">
+        <v>213.4997417926788</v>
+      </c>
+      <c r="G14" t="n">
+        <v>111.015224829452</v>
+      </c>
+      <c r="H14" t="n">
+        <v>51.99782627243387</v>
+      </c>
+      <c r="I14" t="n">
+        <v>135.0001235008241</v>
+      </c>
+      <c r="J14" t="n">
+        <v>291.9993600845335</v>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>low repeatability / inspect</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>2455_a_test/test3/test4 Rx2Tx2 minus Rx1Tx1 offset: CV 52.0%; low repeatability / inspect.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2455_a_test/test3/test4</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>preferred_us</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>preferred US change-point count</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>us_change_points_until_offset_or_last</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>3</v>
+      </c>
+      <c r="F15" t="n">
+        <v>3.666666666666667</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0.5773502691896258</v>
+      </c>
+      <c r="H15" t="n">
+        <v>15.74591643244434</v>
+      </c>
+      <c r="I15" t="n">
+        <v>3</v>
+      </c>
+      <c r="J15" t="n">
+        <v>4</v>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>inspect</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>2455_a_test/test3/test4 preferred US change-point count: CV 15.7%; inspect.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2455_a_test/test3/test4</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>preferred_us</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>preferred US duration</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>us_detachment_duration_s</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>2</v>
+      </c>
+      <c r="F16" t="n">
+        <v>462.0011442899703</v>
+      </c>
+      <c r="G16" t="n">
+        <v>73.53742324697041</v>
+      </c>
+      <c r="H16" t="n">
+        <v>15.91715175510808</v>
+      </c>
+      <c r="I16" t="n">
+        <v>410.0023336410522</v>
+      </c>
+      <c r="J16" t="n">
+        <v>513.9999549388883</v>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>inspect</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>2455_a_test/test3/test4 preferred US duration: CV 15.9%; inspect.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2455_a_test/test3/test4</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>summary duration</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>summary_detachment_duration_s</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>3</v>
+      </c>
+      <c r="F17" t="n">
+        <v>421</v>
+      </c>
+      <c r="G17" t="n">
+        <v>90.14987520790032</v>
+      </c>
+      <c r="H17" t="n">
+        <v>21.41327202087894</v>
+      </c>
+      <c r="I17" t="n">
+        <v>334</v>
+      </c>
+      <c r="J17" t="n">
+        <v>514</v>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>low repeatability / inspect</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>2455_a_test/test3/test4 summary duration: CV 21.4%; low repeatability / inspect.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2455_b/b2/b3/b4</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Rx1Tx1</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Rx1Tx1 change-point count</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>rx1_change_points_until_offset_or_last</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>4</v>
+      </c>
+      <c r="F18" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H18" t="n">
+        <v>22.22222222222222</v>
+      </c>
+      <c r="I18" t="n">
+        <v>2</v>
+      </c>
+      <c r="J18" t="n">
+        <v>3</v>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>low repeatability / inspect</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>2455_b/b2/b3/b4 Rx1Tx1 change-point count: CV 22.2%; low repeatability / inspect.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2455_b/b2/b3/b4</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Rx1Tx1</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Rx1Tx1 duration</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>rx1_detachment_duration_s</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>2</v>
+      </c>
+      <c r="F19" t="n">
+        <v>488.9512953567505</v>
+      </c>
+      <c r="G19" t="n">
+        <v>106.0255002054229</v>
+      </c>
+      <c r="H19" t="n">
+        <v>21.68426614517181</v>
+      </c>
+      <c r="I19" t="n">
+        <v>413.9799451828003</v>
+      </c>
+      <c r="J19" t="n">
+        <v>563.9226455307007</v>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>low repeatability / inspect</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>2455_b/b2/b3/b4 Rx1Tx1 duration: CV 21.7%; low repeatability / inspect.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2455_b/b2/b3/b4</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Rx2Tx2</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Rx2Tx2 change-point count</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>rx2_change_points_until_offset_or_last</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F20" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0.5773502691896257</v>
+      </c>
+      <c r="H20" t="n">
+        <v>38.49001794597505</v>
+      </c>
+      <c r="I20" t="n">
+        <v>1</v>
+      </c>
+      <c r="J20" t="n">
+        <v>2</v>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>low repeatability / inspect</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>2455_b/b2/b3/b4 Rx2Tx2 change-point count: CV 38.5%; low repeatability / inspect.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2455_b/b2/b3/b4</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Rx2Tx2</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Rx2Tx2 duration</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>rx2_detachment_duration_s</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>4</v>
+      </c>
+      <c r="F21" t="n">
+        <v>154.2101740670204</v>
+      </c>
+      <c r="G21" t="n">
+        <v>95.60731284358634</v>
+      </c>
+      <c r="H21" t="n">
+        <v>61.99805779483461</v>
+      </c>
+      <c r="I21" t="n">
+        <v>51.97997832298279</v>
+      </c>
+      <c r="J21" t="n">
+        <v>282.9383995246889</v>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>low repeatability / inspect</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>2455_b/b2/b3/b4 Rx2Tx2 duration: CV 62.0%; low repeatability / inspect.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2455_b/b2/b3/b4</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>channel_difference</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Rx2Tx2 minus Rx1Tx1 offset</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>rx2_minus_rx1_offset_s</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F22" t="n">
+        <v>-385.9999740123749</v>
+      </c>
+      <c r="G22" t="n">
+        <v>31.11270848745182</v>
+      </c>
+      <c r="H22" t="n">
+        <v>8.060287715577504</v>
+      </c>
+      <c r="I22" t="n">
+        <v>-407.9999811649324</v>
+      </c>
+      <c r="J22" t="n">
+        <v>-363.9999668598175</v>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>moderate repeatability</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>2455_b/b2/b3/b4 Rx2Tx2 minus Rx1Tx1 offset: CV 8.1%; moderate repeatability.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2455_b/b2/b3/b4</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>preferred_us</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>preferred US change-point count</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>us_change_points_until_offset_or_last</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>4</v>
+      </c>
+      <c r="F23" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0.5773502691896257</v>
+      </c>
+      <c r="H23" t="n">
+        <v>38.49001794597505</v>
+      </c>
+      <c r="I23" t="n">
+        <v>1</v>
+      </c>
+      <c r="J23" t="n">
+        <v>2</v>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>low repeatability / inspect</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>2455_b/b2/b3/b4 preferred US change-point count: CV 38.5%; low repeatability / inspect.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2455_b/b2/b3/b4</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>preferred_us</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>preferred US duration</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>us_detachment_duration_s</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>4</v>
+      </c>
+      <c r="F24" t="n">
+        <v>154.2101740670204</v>
+      </c>
+      <c r="G24" t="n">
+        <v>95.60731284358634</v>
+      </c>
+      <c r="H24" t="n">
+        <v>61.99805779483461</v>
+      </c>
+      <c r="I24" t="n">
+        <v>51.97997832298279</v>
+      </c>
+      <c r="J24" t="n">
+        <v>282.9383995246889</v>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>low repeatability / inspect</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>2455_b/b2/b3/b4 preferred US duration: CV 62.0%; low repeatability / inspect.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2455_b/b2/b3/b4</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>summary duration</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>summary_detachment_duration_s</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>4</v>
+      </c>
+      <c r="F25" t="n">
+        <v>168.5</v>
+      </c>
+      <c r="G25" t="n">
+        <v>88.63972021616495</v>
+      </c>
+      <c r="H25" t="n">
+        <v>52.60517520247178</v>
+      </c>
+      <c r="I25" t="n">
+        <v>68</v>
+      </c>
+      <c r="J25" t="n">
+        <v>284</v>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>low repeatability / inspect</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>2455_b/b2/b3/b4 summary duration: CV 52.6%; low repeatability / inspect.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2561_a</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Rx1Tx1</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Rx1Tx1 change-point count</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>rx1_change_points_until_offset_or_last</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>2</v>
+      </c>
+      <c r="F26" t="n">
+        <v>4</v>
+      </c>
+      <c r="G26" t="n">
+        <v>1.414213562373095</v>
+      </c>
+      <c r="H26" t="n">
+        <v>35.35533905932738</v>
+      </c>
+      <c r="I26" t="n">
+        <v>3</v>
+      </c>
+      <c r="J26" t="n">
+        <v>5</v>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>low repeatability / inspect</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>2561_a Rx1Tx1 change-point count: CV 35.4%; low repeatability / inspect.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2561_a</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Rx2Tx2</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Rx2Tx2 change-point count</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>rx2_change_points_until_offset_or_last</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>2</v>
+      </c>
+      <c r="F27" t="n">
+        <v>3</v>
+      </c>
+      <c r="G27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" t="n">
+        <v>3</v>
+      </c>
+      <c r="J27" t="n">
+        <v>3</v>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>high repeatability</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>2561_a Rx2Tx2 change-point count: CV 0.0%; high repeatability.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2561_a</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Rx2Tx2</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Rx2Tx2 duration</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>rx2_detachment_duration_s</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>2</v>
+      </c>
+      <c r="F28" t="n">
+        <v>301.4827980995177</v>
+      </c>
+      <c r="G28" t="n">
+        <v>21.94458342977721</v>
+      </c>
+      <c r="H28" t="n">
+        <v>7.278884091600288</v>
+      </c>
+      <c r="I28" t="n">
+        <v>285.9656343460083</v>
+      </c>
+      <c r="J28" t="n">
+        <v>316.9999618530271</v>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>moderate repeatability</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>2561_a Rx2Tx2 duration: CV 7.3%; moderate repeatability.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2561_a</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>preferred_us</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>preferred US change-point count</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>us_change_points_until_offset_or_last</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>2</v>
+      </c>
+      <c r="F29" t="n">
+        <v>3</v>
+      </c>
+      <c r="G29" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" t="n">
+        <v>0</v>
+      </c>
+      <c r="I29" t="n">
+        <v>3</v>
+      </c>
+      <c r="J29" t="n">
+        <v>3</v>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>high repeatability</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>2561_a preferred US change-point count: CV 0.0%; high repeatability.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2561_a</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>preferred_us</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>preferred US duration</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>us_detachment_duration_s</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>2</v>
+      </c>
+      <c r="F30" t="n">
+        <v>301.4827980995177</v>
+      </c>
+      <c r="G30" t="n">
+        <v>21.94458342977721</v>
+      </c>
+      <c r="H30" t="n">
+        <v>7.278884091600288</v>
+      </c>
+      <c r="I30" t="n">
+        <v>285.9656343460083</v>
+      </c>
+      <c r="J30" t="n">
+        <v>316.9999618530271</v>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>moderate repeatability</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>2561_a preferred US duration: CV 7.3%; moderate repeatability.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2561_a</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>summary duration</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>summary_detachment_duration_s</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>2</v>
+      </c>
+      <c r="F31" t="n">
+        <v>326.5</v>
+      </c>
+      <c r="G31" t="n">
+        <v>3.535533905932738</v>
+      </c>
+      <c r="H31" t="n">
+        <v>1.082858776702217</v>
+      </c>
+      <c r="I31" t="n">
+        <v>324</v>
+      </c>
+      <c r="J31" t="n">
+        <v>329</v>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>high repeatability</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>2561_a summary duration: CV 1.1%; high repeatability.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:L31"/>
+  <conditionalFormatting sqref="H2:H31">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="0063BE7B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="00F8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:AB13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -10729,7 +12586,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -15235,11 +17092,23 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:K89"/>
+  <conditionalFormatting sqref="G2:G89">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="0063BE7B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="00F8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -17079,7 +18948,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -18761,117 +20630,4 @@
   <autoFilter ref="A1:P25"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A456"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>2455_a_test_zones_us_offsets.png</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>2455_a_test3_zones_us_offsets.png</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>2455_a_test4_zones_us_offsets.png</t>
-        </is>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" t="inlineStr">
-        <is>
-          <t>2455_a5_zones_us_offsets.png</t>
-        </is>
-      </c>
-    </row>
-    <row r="141">
-      <c r="A141" t="inlineStr">
-        <is>
-          <t>2455_a6_zones_us_offsets.png</t>
-        </is>
-      </c>
-    </row>
-    <row r="176">
-      <c r="A176" t="inlineStr">
-        <is>
-          <t>2455_a7_zones_us_offsets.png</t>
-        </is>
-      </c>
-    </row>
-    <row r="211">
-      <c r="A211" t="inlineStr">
-        <is>
-          <t>2455_b_zones_us_offsets.png</t>
-        </is>
-      </c>
-    </row>
-    <row r="246">
-      <c r="A246" t="inlineStr">
-        <is>
-          <t>2455_b2_zones_us_offsets.png</t>
-        </is>
-      </c>
-    </row>
-    <row r="281">
-      <c r="A281" t="inlineStr">
-        <is>
-          <t>2455_b3_zones_us_offsets.png</t>
-        </is>
-      </c>
-    </row>
-    <row r="316">
-      <c r="A316" t="inlineStr">
-        <is>
-          <t>2455_b4_zones_us_offsets.png</t>
-        </is>
-      </c>
-    </row>
-    <row r="351">
-      <c r="A351" t="inlineStr">
-        <is>
-          <t>2561_a1_zones_us_offsets.png</t>
-        </is>
-      </c>
-    </row>
-    <row r="386">
-      <c r="A386" t="inlineStr">
-        <is>
-          <t>2561_a2_zones_us_offsets.png</t>
-        </is>
-      </c>
-    </row>
-    <row r="421">
-      <c r="A421" t="inlineStr">
-        <is>
-          <t>2561_a3_zones_us_offsets.png</t>
-        </is>
-      </c>
-    </row>
-    <row r="456">
-      <c r="A456" t="inlineStr">
-        <is>
-          <t>2561_a4_zones_us_offsets.png</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Use cooling-relative detachment offsets
</commit_message>
<xml_diff>
--- a/outputs/lab_trials/lab_trials_repeatability_report.xlsx
+++ b/outputs/lab_trials/lab_trials_repeatability_report.xlsx
@@ -28,10 +28,10 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'2 Repeatability CV'!$A$1:$L$41</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'3 Temp Explains Outcomes'!$A$1:$N$33</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'4 Detachment CV'!$A$1:$L$23</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'5 Detachment US Overview'!$A$1:$AA$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'5 Detachment US Overview'!$A$1:$AE$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'6 Detachment Statistics'!$A$1:$K$71</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Raw Sheet Inventory'!$A$1:$K$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Detachment Figure Data'!$A$1:$L$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Detachment Figure Data'!$A$1:$M$25</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'US Rupture Decisions'!$A$1:$R$25</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'US Change Points'!$A$1:$P$25</definedName>
   </definedNames>
@@ -1718,7 +1718,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Duration and offset plots use only full-detachment rows for that sensor. Change-point count plots include available diagnostic counts, including partial rows.</t>
+          <t>Duration and offset plots use only full-detachment rows for that sensor. Offset comparisons are relative to each trial cooling start. Change-point count plots include available diagnostic counts, including partial rows.</t>
         </is>
       </c>
     </row>
@@ -12601,36 +12601,40 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA13"/>
+  <dimension ref="A1:AE13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
-    <col width="32" customWidth="1" min="5" max="5"/>
-    <col width="26" customWidth="1" min="6" max="6"/>
-    <col width="32" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="32" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
     <col width="32" customWidth="1" min="8" max="8"/>
-    <col width="21" customWidth="1" min="9" max="9"/>
-    <col width="32" customWidth="1" min="10" max="10"/>
+    <col width="32" customWidth="1" min="9" max="9"/>
+    <col width="21" customWidth="1" min="10" max="10"/>
     <col width="32" customWidth="1" min="11" max="11"/>
     <col width="32" customWidth="1" min="12" max="12"/>
-    <col width="30" customWidth="1" min="13" max="13"/>
+    <col width="32" customWidth="1" min="13" max="13"/>
     <col width="32" customWidth="1" min="14" max="14"/>
-    <col width="20" customWidth="1" min="15" max="15"/>
-    <col width="27" customWidth="1" min="16" max="16"/>
-    <col width="32" customWidth="1" min="17" max="17"/>
-    <col width="32" customWidth="1" min="18" max="18"/>
-    <col width="20" customWidth="1" min="19" max="19"/>
-    <col width="27" customWidth="1" min="20" max="20"/>
+    <col width="30" customWidth="1" min="15" max="15"/>
+    <col width="32" customWidth="1" min="16" max="16"/>
+    <col width="20" customWidth="1" min="17" max="17"/>
+    <col width="29" customWidth="1" min="18" max="18"/>
+    <col width="27" customWidth="1" min="19" max="19"/>
+    <col width="32" customWidth="1" min="20" max="20"/>
     <col width="32" customWidth="1" min="21" max="21"/>
-    <col width="24" customWidth="1" min="22" max="22"/>
-    <col width="26" customWidth="1" min="23" max="23"/>
-    <col width="32" customWidth="1" min="24" max="24"/>
-    <col width="29" customWidth="1" min="25" max="25"/>
-    <col width="27" customWidth="1" min="26" max="26"/>
-    <col width="32" customWidth="1" min="27" max="27"/>
+    <col width="20" customWidth="1" min="22" max="22"/>
+    <col width="29" customWidth="1" min="23" max="23"/>
+    <col width="27" customWidth="1" min="24" max="24"/>
+    <col width="32" customWidth="1" min="25" max="25"/>
+    <col width="24" customWidth="1" min="26" max="26"/>
+    <col width="26" customWidth="1" min="27" max="27"/>
+    <col width="32" customWidth="1" min="28" max="28"/>
+    <col width="29" customWidth="1" min="29" max="29"/>
+    <col width="27" customWidth="1" min="30" max="30"/>
+    <col width="32" customWidth="1" min="31" max="31"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -12651,120 +12655,140 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>cooling_start_s</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>primary_channel</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>primary_rule</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>summary_sensor_code_used</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>summary_detachment_onset_abs_s</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>primary_detachment_onset_abs_s</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>primary_us_offset_s</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>primary_us_offset_rel_to_cooling_s</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>primary_us_detachment_duration_s</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>primary_us_offset_status</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>primary_us_change_points_until_offset_or_last</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>primary_us_level_at_decision</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>rx1_status</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>rx1_offset_s</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>rx1_offset_rel_to_cooling_s</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>rx1_detachment_duration_s</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>rx1_change_points_until_offset_or_last</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>rx2_status</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>rx2_offset_s</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>rx2_offset_rel_to_cooling_s</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>rx2_detachment_duration_s</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>rx2_change_points_until_offset_or_last</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>rx2_minus_rx1_offset_s</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>rx2_minus_rx1_duration_s</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>complete_detachment_sensor_count</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>complete_detachment_sensors</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>both_channels_full_offset</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>interpretation</t>
         </is>
@@ -12786,90 +12810,102 @@
           <t>at2455_a5</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" t="n">
+        <v>695</v>
+      </c>
+      <c r="E2" t="inlineStr">
         <is>
           <t>Rx2Tx2</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Rx2Tx2 is the primary comparison channel when present; Rx1Tx1 is retained as parallel-sensor validation.</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>22</t>
         </is>
-      </c>
-      <c r="G2" t="n">
-        <v>1000</v>
       </c>
       <c r="H2" t="n">
         <v>1000</v>
       </c>
       <c r="I2" t="n">
+        <v>1000</v>
+      </c>
+      <c r="J2" t="n">
         <v>1219.998578548431</v>
       </c>
-      <c r="J2" t="n">
+      <c r="K2" t="n">
+        <v>524.9985785484312</v>
+      </c>
+      <c r="L2" t="n">
         <v>219.9985785484312</v>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>full_detachment_for_channel</t>
         </is>
       </c>
-      <c r="L2" t="n">
+      <c r="N2" t="n">
         <v>1</v>
       </c>
-      <c r="M2" t="n">
+      <c r="O2" t="n">
         <v>0.5741389473170442</v>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>full_detachment_for_channel</t>
         </is>
       </c>
-      <c r="O2" t="n">
+      <c r="Q2" t="n">
         <v>1665.001210689545</v>
       </c>
-      <c r="P2" t="n">
+      <c r="R2" t="n">
+        <v>970.0012106895447</v>
+      </c>
+      <c r="S2" t="n">
         <v>520.0012106895447</v>
       </c>
-      <c r="Q2" t="n">
+      <c r="T2" t="n">
         <v>2</v>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="U2" t="inlineStr">
         <is>
           <t>full_detachment_for_channel</t>
         </is>
       </c>
-      <c r="S2" t="n">
+      <c r="V2" t="n">
         <v>1219.998578548431</v>
       </c>
-      <c r="T2" t="n">
+      <c r="W2" t="n">
+        <v>524.9985785484312</v>
+      </c>
+      <c r="X2" t="n">
         <v>219.9985785484312</v>
       </c>
-      <c r="U2" t="n">
+      <c r="Y2" t="n">
         <v>1</v>
       </c>
-      <c r="V2" t="n">
+      <c r="Z2" t="n">
         <v>-445.0026321411135</v>
       </c>
-      <c r="W2" t="n">
+      <c r="AA2" t="n">
         <v>-300.0026321411135</v>
       </c>
-      <c r="X2" t="n">
+      <c r="AB2" t="n">
         <v>2</v>
       </c>
-      <c r="Y2" t="inlineStr">
+      <c r="AC2" t="inlineStr">
         <is>
           <t>Rx1Tx1, Rx2Tx2</t>
         </is>
       </c>
-      <c r="Z2" t="n">
+      <c r="AD2" t="n">
         <v>1</v>
       </c>
-      <c r="AA2" t="inlineStr">
+      <c r="AE2" t="inlineStr">
         <is>
           <t>2455_a5: 2 sensor(s) reached full US detachment (Rx1Tx1, Rx2Tx2). Rx2 minus Rx1 offset = -445.0 s.</t>
         </is>
@@ -12891,90 +12927,102 @@
           <t>at2455_a6</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" t="n">
+        <v>1285</v>
+      </c>
+      <c r="E3" t="inlineStr">
         <is>
           <t>Rx2Tx2</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>Rx2Tx2 is the primary comparison channel when present; Rx1Tx1 is retained as parallel-sensor validation.</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>22</t>
         </is>
-      </c>
-      <c r="G3" t="n">
-        <v>1630</v>
       </c>
       <c r="H3" t="n">
         <v>1630</v>
       </c>
       <c r="I3" t="n">
+        <v>1630</v>
+      </c>
+      <c r="J3" t="n">
         <v>1880.000734806061</v>
       </c>
-      <c r="J3" t="n">
+      <c r="K3" t="n">
+        <v>595.0007348060608</v>
+      </c>
+      <c r="L3" t="n">
         <v>250.0007348060608</v>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>full_detachment_for_channel</t>
         </is>
       </c>
-      <c r="L3" t="n">
+      <c r="N3" t="n">
         <v>1</v>
       </c>
-      <c r="M3" t="n">
+      <c r="O3" t="n">
         <v>0.5454090153670035</v>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t>full_detachment_for_channel</t>
         </is>
       </c>
-      <c r="O3" t="n">
+      <c r="Q3" t="n">
         <v>2415.000879526138</v>
       </c>
-      <c r="P3" t="n">
+      <c r="R3" t="n">
+        <v>1130.000879526138</v>
+      </c>
+      <c r="S3" t="n">
         <v>655.0008795261383</v>
       </c>
-      <c r="Q3" t="n">
+      <c r="T3" t="n">
         <v>3</v>
       </c>
-      <c r="R3" t="inlineStr">
+      <c r="U3" t="inlineStr">
         <is>
           <t>full_detachment_for_channel</t>
         </is>
       </c>
-      <c r="S3" t="n">
+      <c r="V3" t="n">
         <v>1880.000734806061</v>
       </c>
-      <c r="T3" t="n">
+      <c r="W3" t="n">
+        <v>595.0007348060608</v>
+      </c>
+      <c r="X3" t="n">
         <v>250.0007348060608</v>
       </c>
-      <c r="U3" t="n">
+      <c r="Y3" t="n">
         <v>1</v>
       </c>
-      <c r="V3" t="n">
+      <c r="Z3" t="n">
         <v>-535.0001447200775</v>
       </c>
-      <c r="W3" t="n">
+      <c r="AA3" t="n">
         <v>-405.0001447200775</v>
       </c>
-      <c r="X3" t="n">
+      <c r="AB3" t="n">
         <v>2</v>
       </c>
-      <c r="Y3" t="inlineStr">
+      <c r="AC3" t="inlineStr">
         <is>
           <t>Rx1Tx1, Rx2Tx2</t>
         </is>
       </c>
-      <c r="Z3" t="n">
+      <c r="AD3" t="n">
         <v>1</v>
       </c>
-      <c r="AA3" t="inlineStr">
+      <c r="AE3" t="inlineStr">
         <is>
           <t>2455_a6: 2 sensor(s) reached full US detachment (Rx1Tx1, Rx2Tx2). Rx2 minus Rx1 offset = -535.0 s.</t>
         </is>
@@ -12996,90 +13044,102 @@
           <t>at2455_a7</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" t="n">
+        <v>660</v>
+      </c>
+      <c r="E4" t="inlineStr">
         <is>
           <t>Rx2Tx2</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>Rx2Tx2 is the primary comparison channel when present; Rx1Tx1 is retained as parallel-sensor validation.</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>22</t>
         </is>
-      </c>
-      <c r="G4" t="n">
-        <v>985</v>
       </c>
       <c r="H4" t="n">
         <v>985</v>
       </c>
       <c r="I4" t="n">
+        <v>985</v>
+      </c>
+      <c r="J4" t="n">
         <v>1325.000415086746</v>
       </c>
-      <c r="J4" t="n">
+      <c r="K4" t="n">
+        <v>665.0004150867462</v>
+      </c>
+      <c r="L4" t="n">
         <v>340.0004150867462</v>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>full_detachment_for_channel</t>
         </is>
       </c>
-      <c r="L4" t="n">
+      <c r="N4" t="n">
         <v>3</v>
       </c>
-      <c r="M4" t="n">
+      <c r="O4" t="n">
         <v>0.8325951321135664</v>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="P4" t="inlineStr">
         <is>
           <t>full_detachment_for_channel</t>
         </is>
       </c>
-      <c r="O4" t="n">
+      <c r="Q4" t="n">
         <v>1615.002419471741</v>
       </c>
-      <c r="P4" t="n">
+      <c r="R4" t="n">
+        <v>955.0024194717407</v>
+      </c>
+      <c r="S4" t="n">
         <v>510.0024194717407</v>
       </c>
-      <c r="Q4" t="n">
+      <c r="T4" t="n">
         <v>3</v>
       </c>
-      <c r="R4" t="inlineStr">
+      <c r="U4" t="inlineStr">
         <is>
           <t>full_detachment_for_channel</t>
         </is>
       </c>
-      <c r="S4" t="n">
+      <c r="V4" t="n">
         <v>1325.000415086746</v>
       </c>
-      <c r="T4" t="n">
+      <c r="W4" t="n">
+        <v>665.0004150867462</v>
+      </c>
+      <c r="X4" t="n">
         <v>340.0004150867462</v>
       </c>
-      <c r="U4" t="n">
+      <c r="Y4" t="n">
         <v>3</v>
       </c>
-      <c r="V4" t="n">
+      <c r="Z4" t="n">
         <v>-290.0020043849945</v>
       </c>
-      <c r="W4" t="n">
+      <c r="AA4" t="n">
         <v>-170.0020043849945</v>
       </c>
-      <c r="X4" t="n">
+      <c r="AB4" t="n">
         <v>2</v>
       </c>
-      <c r="Y4" t="inlineStr">
+      <c r="AC4" t="inlineStr">
         <is>
           <t>Rx1Tx1, Rx2Tx2</t>
         </is>
       </c>
-      <c r="Z4" t="n">
+      <c r="AD4" t="n">
         <v>1</v>
       </c>
-      <c r="AA4" t="inlineStr">
+      <c r="AE4" t="inlineStr">
         <is>
           <t>2455_a7: 2 sensor(s) reached full US detachment (Rx1Tx1, Rx2Tx2). Rx2 minus Rx1 offset = -290.0 s.</t>
         </is>
@@ -13101,90 +13161,102 @@
           <t>at2455_a_test</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" t="n">
+        <v>210</v>
+      </c>
+      <c r="E5" t="inlineStr">
         <is>
           <t>Rx2Tx2</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>Rx2Tx2 is the primary comparison channel when present; Rx1Tx1 is retained as parallel-sensor validation.</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>22</t>
         </is>
-      </c>
-      <c r="G5" t="n">
-        <v>595</v>
       </c>
       <c r="H5" t="n">
         <v>595</v>
       </c>
       <c r="I5" t="n">
+        <v>595</v>
+      </c>
+      <c r="J5" t="n">
         <v>1005.002333641052</v>
       </c>
-      <c r="J5" t="n">
+      <c r="K5" t="n">
+        <v>795.0023336410522</v>
+      </c>
+      <c r="L5" t="n">
         <v>410.0023336410522</v>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>full_detachment_for_channel</t>
         </is>
       </c>
-      <c r="L5" t="n">
+      <c r="N5" t="n">
         <v>4</v>
       </c>
-      <c r="M5" t="n">
+      <c r="O5" t="n">
         <v>0.5637620750490631</v>
       </c>
-      <c r="N5" t="inlineStr">
+      <c r="P5" t="inlineStr">
         <is>
           <t>full_detachment_for_channel</t>
         </is>
       </c>
-      <c r="O5" t="n">
+      <c r="Q5" t="n">
         <v>870.0022101402282</v>
       </c>
-      <c r="P5" t="n">
+      <c r="R5" t="n">
+        <v>660.0022101402282</v>
+      </c>
+      <c r="S5" t="n">
         <v>270.0022101402282</v>
       </c>
-      <c r="Q5" t="n">
+      <c r="T5" t="n">
         <v>2</v>
       </c>
-      <c r="R5" t="inlineStr">
+      <c r="U5" t="inlineStr">
         <is>
           <t>full_detachment_for_channel</t>
         </is>
       </c>
-      <c r="S5" t="n">
+      <c r="V5" t="n">
         <v>1005.002333641052</v>
       </c>
-      <c r="T5" t="n">
+      <c r="W5" t="n">
+        <v>795.0023336410522</v>
+      </c>
+      <c r="X5" t="n">
         <v>410.0023336410522</v>
       </c>
-      <c r="U5" t="n">
+      <c r="Y5" t="n">
         <v>4</v>
       </c>
-      <c r="V5" t="n">
+      <c r="Z5" t="n">
         <v>135.0001235008241</v>
       </c>
-      <c r="W5" t="n">
+      <c r="AA5" t="n">
         <v>140.0001235008241</v>
       </c>
-      <c r="X5" t="n">
+      <c r="AB5" t="n">
         <v>2</v>
       </c>
-      <c r="Y5" t="inlineStr">
+      <c r="AC5" t="inlineStr">
         <is>
           <t>Rx1Tx1, Rx2Tx2</t>
         </is>
       </c>
-      <c r="Z5" t="n">
+      <c r="AD5" t="n">
         <v>1</v>
       </c>
-      <c r="AA5" t="inlineStr">
+      <c r="AE5" t="inlineStr">
         <is>
           <t>2455_a_test: 2 sensor(s) reached full US detachment (Rx1Tx1, Rx2Tx2). Rx2 minus Rx1 offset = 135.0 s.</t>
         </is>
@@ -13206,90 +13278,102 @@
           <t>at2455_a_test3</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" t="n">
+        <v>155</v>
+      </c>
+      <c r="E6" t="inlineStr">
         <is>
           <t>Rx2Tx2</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>Rx2Tx2 is the primary comparison channel when present; Rx1Tx1 is retained as parallel-sensor validation.</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>22</t>
         </is>
-      </c>
-      <c r="G6" t="n">
-        <v>479</v>
       </c>
       <c r="H6" t="n">
         <v>479</v>
       </c>
       <c r="I6" t="n">
+        <v>479</v>
+      </c>
+      <c r="J6" t="n">
         <v>992.9999549388883</v>
       </c>
-      <c r="J6" t="n">
+      <c r="K6" t="n">
+        <v>837.9999549388883</v>
+      </c>
+      <c r="L6" t="n">
         <v>513.9999549388883</v>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="M6" t="inlineStr">
         <is>
           <t>full_detachment_for_channel</t>
         </is>
       </c>
-      <c r="L6" t="n">
+      <c r="N6" t="n">
         <v>4</v>
       </c>
-      <c r="M6" t="n">
+      <c r="O6" t="n">
         <v>0.699081120081692</v>
       </c>
-      <c r="N6" t="inlineStr">
+      <c r="P6" t="inlineStr">
         <is>
           <t>full_detachment_for_channel</t>
         </is>
       </c>
-      <c r="O6" t="n">
+      <c r="Q6" t="n">
         <v>701.0005948543549</v>
       </c>
-      <c r="P6" t="n">
+      <c r="R6" t="n">
+        <v>546.0005948543549</v>
+      </c>
+      <c r="S6" t="n">
         <v>206.0005948543549</v>
       </c>
-      <c r="Q6" t="n">
+      <c r="T6" t="n">
         <v>2</v>
       </c>
-      <c r="R6" t="inlineStr">
+      <c r="U6" t="inlineStr">
         <is>
           <t>full_detachment_for_channel</t>
         </is>
       </c>
-      <c r="S6" t="n">
+      <c r="V6" t="n">
         <v>992.9999549388883</v>
       </c>
-      <c r="T6" t="n">
+      <c r="W6" t="n">
+        <v>837.9999549388883</v>
+      </c>
+      <c r="X6" t="n">
         <v>513.9999549388883</v>
       </c>
-      <c r="U6" t="n">
+      <c r="Y6" t="n">
         <v>4</v>
       </c>
-      <c r="V6" t="n">
+      <c r="Z6" t="n">
         <v>291.9993600845335</v>
       </c>
-      <c r="W6" t="n">
+      <c r="AA6" t="n">
         <v>307.9993600845335</v>
       </c>
-      <c r="X6" t="n">
+      <c r="AB6" t="n">
         <v>2</v>
       </c>
-      <c r="Y6" t="inlineStr">
+      <c r="AC6" t="inlineStr">
         <is>
           <t>Rx1Tx1, Rx2Tx2</t>
         </is>
       </c>
-      <c r="Z6" t="n">
+      <c r="AD6" t="n">
         <v>1</v>
       </c>
-      <c r="AA6" t="inlineStr">
+      <c r="AE6" t="inlineStr">
         <is>
           <t>2455_a_test3: 2 sensor(s) reached full US detachment (Rx1Tx1, Rx2Tx2). Rx2 minus Rx1 offset = 292.0 s.</t>
         </is>
@@ -13311,72 +13395,78 @@
           <t>at2455_a_test4</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" t="n">
+        <v>728</v>
+      </c>
+      <c r="E7" t="inlineStr">
         <is>
           <t>Rx2Tx2</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>Rx2Tx2 is the primary comparison channel when present; Rx1Tx1 is retained as parallel-sensor validation.</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>22</t>
         </is>
-      </c>
-      <c r="G7" t="n">
-        <v>1064</v>
       </c>
       <c r="H7" t="n">
         <v>1064</v>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="I7" t="n">
+        <v>1064</v>
+      </c>
+      <c r="M7" t="inlineStr">
         <is>
           <t>partial_detachment_no_change_point_met_threshold</t>
         </is>
       </c>
-      <c r="L7" t="n">
+      <c r="N7" t="n">
         <v>3</v>
       </c>
-      <c r="M7" t="n">
+      <c r="O7" t="n">
         <v>0.485939799054226</v>
       </c>
-      <c r="N7" t="inlineStr">
+      <c r="P7" t="inlineStr">
         <is>
           <t>full_detachment_for_channel</t>
         </is>
       </c>
-      <c r="O7" t="n">
+      <c r="Q7" t="n">
         <v>1289.999727010727</v>
       </c>
-      <c r="P7" t="n">
+      <c r="R7" t="n">
+        <v>561.9997270107267</v>
+      </c>
+      <c r="S7" t="n">
         <v>211.9997270107267</v>
       </c>
-      <c r="Q7" t="n">
+      <c r="T7" t="n">
         <v>2</v>
       </c>
-      <c r="R7" t="inlineStr">
+      <c r="U7" t="inlineStr">
         <is>
           <t>partial_detachment_no_change_point_met_threshold</t>
         </is>
       </c>
-      <c r="U7" t="n">
+      <c r="Y7" t="n">
         <v>3</v>
       </c>
-      <c r="X7" t="n">
+      <c r="AB7" t="n">
         <v>1</v>
       </c>
-      <c r="Y7" t="inlineStr">
+      <c r="AC7" t="inlineStr">
         <is>
           <t>Rx1Tx1</t>
         </is>
       </c>
-      <c r="Z7" t="n">
+      <c r="AD7" t="n">
         <v>0</v>
       </c>
-      <c r="AA7" t="inlineStr">
+      <c r="AE7" t="inlineStr">
         <is>
           <t>2455_a_test4: 1 sensor(s) reached full US detachment (Rx1Tx1). Rx2 minus Rx1 offset = n/a s.</t>
         </is>
@@ -13398,78 +13488,87 @@
           <t>at2455_b</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" t="n">
+        <v>406</v>
+      </c>
+      <c r="E8" t="inlineStr">
         <is>
           <t>Rx2Tx2</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>Rx2Tx2 is the primary comparison channel when present; Rx1Tx1 is retained as parallel-sensor validation.</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>22</t>
         </is>
-      </c>
-      <c r="G8" t="n">
-        <v>1082</v>
       </c>
       <c r="H8" t="n">
         <v>1082</v>
       </c>
       <c r="I8" t="n">
+        <v>1082</v>
+      </c>
+      <c r="J8" t="n">
         <v>1217.999654054641</v>
       </c>
-      <c r="J8" t="n">
+      <c r="K8" t="n">
+        <v>811.9996540546415</v>
+      </c>
+      <c r="L8" t="n">
         <v>135.9996540546415</v>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="M8" t="inlineStr">
         <is>
           <t>full_detachment_for_channel</t>
         </is>
       </c>
-      <c r="L8" t="n">
+      <c r="N8" t="n">
         <v>2</v>
       </c>
-      <c r="M8" t="n">
+      <c r="O8" t="n">
         <v>0.6549491860507034</v>
       </c>
-      <c r="N8" t="inlineStr">
+      <c r="P8" t="inlineStr">
         <is>
           <t>partial_detachment_no_change_point_met_threshold</t>
         </is>
       </c>
-      <c r="Q8" t="n">
+      <c r="T8" t="n">
         <v>2</v>
       </c>
-      <c r="R8" t="inlineStr">
+      <c r="U8" t="inlineStr">
         <is>
           <t>full_detachment_for_channel</t>
         </is>
       </c>
-      <c r="S8" t="n">
+      <c r="V8" t="n">
         <v>1217.999654054641</v>
       </c>
-      <c r="T8" t="n">
+      <c r="W8" t="n">
+        <v>811.9996540546415</v>
+      </c>
+      <c r="X8" t="n">
         <v>135.9996540546415</v>
       </c>
-      <c r="U8" t="n">
+      <c r="Y8" t="n">
         <v>2</v>
       </c>
-      <c r="X8" t="n">
+      <c r="AB8" t="n">
         <v>1</v>
       </c>
-      <c r="Y8" t="inlineStr">
+      <c r="AC8" t="inlineStr">
         <is>
           <t>Rx2Tx2</t>
         </is>
       </c>
-      <c r="Z8" t="n">
+      <c r="AD8" t="n">
         <v>0</v>
       </c>
-      <c r="AA8" t="inlineStr">
+      <c r="AE8" t="inlineStr">
         <is>
           <t>2455_b: 1 sensor(s) reached full US detachment (Rx2Tx2). Rx2 minus Rx1 offset = n/a s.</t>
         </is>
@@ -13491,78 +13590,87 @@
           <t>at2455_b2</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" t="n">
+        <v>217</v>
+      </c>
+      <c r="E9" t="inlineStr">
         <is>
           <t>Rx2Tx2</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>Rx2Tx2 is the primary comparison channel when present; Rx1Tx1 is retained as parallel-sensor validation.</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>22</t>
         </is>
-      </c>
-      <c r="G9" t="n">
-        <v>673.03</v>
       </c>
       <c r="H9" t="n">
         <v>673.03</v>
       </c>
       <c r="I9" t="n">
+        <v>673.03</v>
+      </c>
+      <c r="J9" t="n">
         <v>955.9683995246888</v>
       </c>
-      <c r="J9" t="n">
+      <c r="K9" t="n">
+        <v>738.9683995246888</v>
+      </c>
+      <c r="L9" t="n">
         <v>282.9383995246889</v>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="M9" t="inlineStr">
         <is>
           <t>full_detachment_for_channel</t>
         </is>
       </c>
-      <c r="L9" t="n">
+      <c r="N9" t="n">
         <v>2</v>
       </c>
-      <c r="M9" t="n">
+      <c r="O9" t="n">
         <v>0.7775187872829324</v>
       </c>
-      <c r="N9" t="inlineStr">
+      <c r="P9" t="inlineStr">
         <is>
           <t>partial_detachment_no_change_point_met_threshold</t>
         </is>
       </c>
-      <c r="Q9" t="n">
+      <c r="T9" t="n">
         <v>3</v>
       </c>
-      <c r="R9" t="inlineStr">
+      <c r="U9" t="inlineStr">
         <is>
           <t>full_detachment_for_channel</t>
         </is>
       </c>
-      <c r="S9" t="n">
+      <c r="V9" t="n">
         <v>955.9683995246888</v>
       </c>
-      <c r="T9" t="n">
+      <c r="W9" t="n">
+        <v>738.9683995246888</v>
+      </c>
+      <c r="X9" t="n">
         <v>282.9383995246889</v>
       </c>
-      <c r="U9" t="n">
+      <c r="Y9" t="n">
         <v>2</v>
       </c>
-      <c r="X9" t="n">
+      <c r="AB9" t="n">
         <v>1</v>
       </c>
-      <c r="Y9" t="inlineStr">
+      <c r="AC9" t="inlineStr">
         <is>
           <t>Rx2Tx2</t>
         </is>
       </c>
-      <c r="Z9" t="n">
+      <c r="AD9" t="n">
         <v>0</v>
       </c>
-      <c r="AA9" t="inlineStr">
+      <c r="AE9" t="inlineStr">
         <is>
           <t>2455_b2: 1 sensor(s) reached full US detachment (Rx2Tx2). Rx2 minus Rx1 offset = n/a s.</t>
         </is>
@@ -13584,90 +13692,102 @@
           <t>at2455_b3</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" t="n">
+        <v>162</v>
+      </c>
+      <c r="E10" t="inlineStr">
         <is>
           <t>Rx2Tx2</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>Rx2Tx2 is the primary comparison channel when present; Rx1Tx1 is retained as parallel-sensor validation.</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>22</t>
         </is>
-      </c>
-      <c r="G10" t="n">
-        <v>998</v>
       </c>
       <c r="H10" t="n">
         <v>998</v>
       </c>
       <c r="I10" t="n">
+        <v>998</v>
+      </c>
+      <c r="J10" t="n">
         <v>1049.979978322983</v>
       </c>
-      <c r="J10" t="n">
+      <c r="K10" t="n">
+        <v>887.9799783229828</v>
+      </c>
+      <c r="L10" t="n">
         <v>51.97997832298279</v>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="M10" t="inlineStr">
         <is>
           <t>full_detachment_for_channel</t>
         </is>
       </c>
-      <c r="L10" t="n">
+      <c r="N10" t="n">
         <v>1</v>
       </c>
-      <c r="M10" t="n">
+      <c r="O10" t="n">
         <v>0.7454181265800934</v>
       </c>
-      <c r="N10" t="inlineStr">
+      <c r="P10" t="inlineStr">
         <is>
           <t>full_detachment_for_channel</t>
         </is>
       </c>
-      <c r="O10" t="n">
+      <c r="Q10" t="n">
         <v>1413.9799451828</v>
       </c>
-      <c r="P10" t="n">
+      <c r="R10" t="n">
+        <v>1251.9799451828</v>
+      </c>
+      <c r="S10" t="n">
         <v>413.9799451828003</v>
       </c>
-      <c r="Q10" t="n">
+      <c r="T10" t="n">
         <v>2</v>
       </c>
-      <c r="R10" t="inlineStr">
+      <c r="U10" t="inlineStr">
         <is>
           <t>full_detachment_for_channel</t>
         </is>
       </c>
-      <c r="S10" t="n">
+      <c r="V10" t="n">
         <v>1049.979978322983</v>
       </c>
-      <c r="T10" t="n">
+      <c r="W10" t="n">
+        <v>887.9799783229828</v>
+      </c>
+      <c r="X10" t="n">
         <v>51.97997832298279</v>
       </c>
-      <c r="U10" t="n">
+      <c r="Y10" t="n">
         <v>1</v>
       </c>
-      <c r="V10" t="n">
+      <c r="Z10" t="n">
         <v>-363.9999668598175</v>
       </c>
-      <c r="W10" t="n">
+      <c r="AA10" t="n">
         <v>-361.9999668598175</v>
       </c>
-      <c r="X10" t="n">
+      <c r="AB10" t="n">
         <v>2</v>
       </c>
-      <c r="Y10" t="inlineStr">
+      <c r="AC10" t="inlineStr">
         <is>
           <t>Rx1Tx1, Rx2Tx2</t>
         </is>
       </c>
-      <c r="Z10" t="n">
+      <c r="AD10" t="n">
         <v>1</v>
       </c>
-      <c r="AA10" t="inlineStr">
+      <c r="AE10" t="inlineStr">
         <is>
           <t>2455_b3: 2 sensor(s) reached full US detachment (Rx1Tx1, Rx2Tx2). Rx2 minus Rx1 offset = -364.0 s.</t>
         </is>
@@ -13689,90 +13809,102 @@
           <t>at2455_b4</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" t="n">
+        <v>228</v>
+      </c>
+      <c r="E11" t="inlineStr">
         <is>
           <t>Rx2Tx2</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>Rx2Tx2 is the primary comparison channel when present; Rx1Tx1 is retained as parallel-sensor validation.</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>22</t>
         </is>
-      </c>
-      <c r="G11" t="n">
-        <v>810.04</v>
       </c>
       <c r="H11" t="n">
         <v>810.04</v>
       </c>
       <c r="I11" t="n">
+        <v>810.04</v>
+      </c>
+      <c r="J11" t="n">
         <v>955.9626643657683</v>
       </c>
-      <c r="J11" t="n">
+      <c r="K11" t="n">
+        <v>727.9626643657683</v>
+      </c>
+      <c r="L11" t="n">
         <v>145.9226643657684</v>
       </c>
-      <c r="K11" t="inlineStr">
+      <c r="M11" t="inlineStr">
         <is>
           <t>full_detachment_for_channel</t>
         </is>
       </c>
-      <c r="L11" t="n">
+      <c r="N11" t="n">
         <v>1</v>
       </c>
-      <c r="M11" t="n">
+      <c r="O11" t="n">
         <v>0.8044727888986035</v>
       </c>
-      <c r="N11" t="inlineStr">
+      <c r="P11" t="inlineStr">
         <is>
           <t>full_detachment_for_channel</t>
         </is>
       </c>
-      <c r="O11" t="n">
+      <c r="Q11" t="n">
         <v>1363.962645530701</v>
       </c>
-      <c r="P11" t="n">
+      <c r="R11" t="n">
+        <v>1135.962645530701</v>
+      </c>
+      <c r="S11" t="n">
         <v>563.9226455307007</v>
       </c>
-      <c r="Q11" t="n">
+      <c r="T11" t="n">
         <v>2</v>
       </c>
-      <c r="R11" t="inlineStr">
+      <c r="U11" t="inlineStr">
         <is>
           <t>full_detachment_for_channel</t>
         </is>
       </c>
-      <c r="S11" t="n">
+      <c r="V11" t="n">
         <v>955.9626643657683</v>
       </c>
-      <c r="T11" t="n">
+      <c r="W11" t="n">
+        <v>727.9626643657683</v>
+      </c>
+      <c r="X11" t="n">
         <v>145.9226643657684</v>
       </c>
-      <c r="U11" t="n">
+      <c r="Y11" t="n">
         <v>1</v>
       </c>
-      <c r="V11" t="n">
+      <c r="Z11" t="n">
         <v>-407.9999811649324</v>
       </c>
-      <c r="W11" t="n">
+      <c r="AA11" t="n">
         <v>-417.9999811649324</v>
       </c>
-      <c r="X11" t="n">
+      <c r="AB11" t="n">
         <v>2</v>
       </c>
-      <c r="Y11" t="inlineStr">
+      <c r="AC11" t="inlineStr">
         <is>
           <t>Rx1Tx1, Rx2Tx2</t>
         </is>
       </c>
-      <c r="Z11" t="n">
+      <c r="AD11" t="n">
         <v>1</v>
       </c>
-      <c r="AA11" t="inlineStr">
+      <c r="AE11" t="inlineStr">
         <is>
           <t>2455_b4: 2 sensor(s) reached full US detachment (Rx1Tx1, Rx2Tx2). Rx2 minus Rx1 offset = -408.0 s.</t>
         </is>
@@ -13794,78 +13926,87 @@
           <t>at2561_a3</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D12" t="n">
+        <v>660</v>
+      </c>
+      <c r="E12" t="inlineStr">
         <is>
           <t>Rx2Tx2</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>Rx2Tx2 is the primary comparison channel when present; Rx1Tx1 is retained as parallel-sensor validation.</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>22</t>
         </is>
-      </c>
-      <c r="G12" t="n">
-        <v>1076</v>
       </c>
       <c r="H12" t="n">
         <v>1076</v>
       </c>
       <c r="I12" t="n">
+        <v>1076</v>
+      </c>
+      <c r="J12" t="n">
         <v>1361.965634346008</v>
       </c>
-      <c r="J12" t="n">
+      <c r="K12" t="n">
+        <v>701.9656343460083</v>
+      </c>
+      <c r="L12" t="n">
         <v>285.9656343460083</v>
       </c>
-      <c r="K12" t="inlineStr">
+      <c r="M12" t="inlineStr">
         <is>
           <t>full_detachment_for_channel</t>
         </is>
       </c>
-      <c r="L12" t="n">
+      <c r="N12" t="n">
         <v>3</v>
       </c>
-      <c r="M12" t="n">
+      <c r="O12" t="n">
         <v>0.7621613005628776</v>
       </c>
-      <c r="N12" t="inlineStr">
+      <c r="P12" t="inlineStr">
         <is>
           <t>partial_detachment_no_change_point_met_threshold</t>
         </is>
       </c>
-      <c r="Q12" t="n">
+      <c r="T12" t="n">
         <v>5</v>
       </c>
-      <c r="R12" t="inlineStr">
+      <c r="U12" t="inlineStr">
         <is>
           <t>full_detachment_for_channel</t>
         </is>
       </c>
-      <c r="S12" t="n">
+      <c r="V12" t="n">
         <v>1361.965634346008</v>
       </c>
-      <c r="T12" t="n">
+      <c r="W12" t="n">
+        <v>701.9656343460083</v>
+      </c>
+      <c r="X12" t="n">
         <v>285.9656343460083</v>
       </c>
-      <c r="U12" t="n">
+      <c r="Y12" t="n">
         <v>3</v>
       </c>
-      <c r="X12" t="n">
+      <c r="AB12" t="n">
         <v>1</v>
       </c>
-      <c r="Y12" t="inlineStr">
+      <c r="AC12" t="inlineStr">
         <is>
           <t>Rx2Tx2</t>
         </is>
       </c>
-      <c r="Z12" t="n">
+      <c r="AD12" t="n">
         <v>0</v>
       </c>
-      <c r="AA12" t="inlineStr">
+      <c r="AE12" t="inlineStr">
         <is>
           <t>2561_a3: 1 sensor(s) reached full US detachment (Rx2Tx2). Rx2 minus Rx1 offset = n/a s.</t>
         </is>
@@ -13887,85 +14028,94 @@
           <t>at2561_a4</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D13" t="n">
+        <v>645</v>
+      </c>
+      <c r="E13" t="inlineStr">
         <is>
           <t>Rx2Tx2</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>Rx2Tx2 is the primary comparison channel when present; Rx1Tx1 is retained as parallel-sensor validation.</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="G13" t="inlineStr">
         <is>
           <t>22</t>
         </is>
-      </c>
-      <c r="G13" t="n">
-        <v>1033</v>
       </c>
       <c r="H13" t="n">
         <v>1033</v>
       </c>
       <c r="I13" t="n">
+        <v>1033</v>
+      </c>
+      <c r="J13" t="n">
         <v>1349.999961853027</v>
       </c>
-      <c r="J13" t="n">
+      <c r="K13" t="n">
+        <v>704.9999618530271</v>
+      </c>
+      <c r="L13" t="n">
         <v>316.9999618530271</v>
       </c>
-      <c r="K13" t="inlineStr">
+      <c r="M13" t="inlineStr">
         <is>
           <t>full_detachment_for_channel</t>
         </is>
       </c>
-      <c r="L13" t="n">
+      <c r="N13" t="n">
         <v>3</v>
       </c>
-      <c r="M13" t="n">
+      <c r="O13" t="n">
         <v>0.7769129392553277</v>
       </c>
-      <c r="N13" t="inlineStr">
+      <c r="P13" t="inlineStr">
         <is>
           <t>partial_detachment_no_change_point_met_threshold</t>
         </is>
       </c>
-      <c r="Q13" t="n">
+      <c r="T13" t="n">
         <v>3</v>
       </c>
-      <c r="R13" t="inlineStr">
+      <c r="U13" t="inlineStr">
         <is>
           <t>full_detachment_for_channel</t>
         </is>
       </c>
-      <c r="S13" t="n">
+      <c r="V13" t="n">
         <v>1349.999961853027</v>
       </c>
-      <c r="T13" t="n">
+      <c r="W13" t="n">
+        <v>704.9999618530271</v>
+      </c>
+      <c r="X13" t="n">
         <v>316.9999618530271</v>
       </c>
-      <c r="U13" t="n">
+      <c r="Y13" t="n">
         <v>3</v>
       </c>
-      <c r="X13" t="n">
+      <c r="AB13" t="n">
         <v>1</v>
       </c>
-      <c r="Y13" t="inlineStr">
+      <c r="AC13" t="inlineStr">
         <is>
           <t>Rx2Tx2</t>
         </is>
       </c>
-      <c r="Z13" t="n">
+      <c r="AD13" t="n">
         <v>0</v>
       </c>
-      <c r="AA13" t="inlineStr">
+      <c r="AE13" t="inlineStr">
         <is>
           <t>2561_a4: 1 sensor(s) reached full US detachment (Rx2Tx2). Rx2 minus Rx1 offset = n/a s.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AA13"/>
+  <autoFilter ref="A1:AE13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -18361,7 +18511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L25"/>
+  <dimension ref="A1:M25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -18372,10 +18522,11 @@
     <col width="32" customWidth="1" min="6" max="6"/>
     <col width="32" customWidth="1" min="7" max="7"/>
     <col width="23" customWidth="1" min="8" max="8"/>
-    <col width="21" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
     <col width="32" customWidth="1" min="10" max="10"/>
     <col width="32" customWidth="1" min="11" max="11"/>
     <col width="32" customWidth="1" min="12" max="12"/>
+    <col width="32" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -18421,20 +18572,25 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>detachment_offset_s</t>
+          <t>detachment_offset_absolute_s</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
+          <t>detachment_offset_rel_to_cooling_s</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t>change_points_until_offset_or_last</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>complete_detachment_sensor_count_for_rep</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>complete_detachment_sensors_for_rep</t>
         </is>
@@ -18479,12 +18635,15 @@
         <v>1665.001210689545</v>
       </c>
       <c r="J2" t="n">
-        <v>2</v>
+        <v>970.0012106895447</v>
       </c>
       <c r="K2" t="n">
         <v>2</v>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="L2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M2" t="inlineStr">
         <is>
           <t>Rx1Tx1, Rx2Tx2</t>
         </is>
@@ -18529,12 +18688,15 @@
         <v>1219.998578548431</v>
       </c>
       <c r="J3" t="n">
+        <v>524.9985785484312</v>
+      </c>
+      <c r="K3" t="n">
         <v>1</v>
       </c>
-      <c r="K3" t="n">
+      <c r="L3" t="n">
         <v>2</v>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>Rx1Tx1, Rx2Tx2</t>
         </is>
@@ -18579,12 +18741,15 @@
         <v>2415.000879526138</v>
       </c>
       <c r="J4" t="n">
+        <v>1130.000879526138</v>
+      </c>
+      <c r="K4" t="n">
         <v>3</v>
       </c>
-      <c r="K4" t="n">
+      <c r="L4" t="n">
         <v>2</v>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>Rx1Tx1, Rx2Tx2</t>
         </is>
@@ -18629,12 +18794,15 @@
         <v>1880.000734806061</v>
       </c>
       <c r="J5" t="n">
+        <v>595.0007348060608</v>
+      </c>
+      <c r="K5" t="n">
         <v>1</v>
       </c>
-      <c r="K5" t="n">
+      <c r="L5" t="n">
         <v>2</v>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>Rx1Tx1, Rx2Tx2</t>
         </is>
@@ -18679,12 +18847,15 @@
         <v>1615.002419471741</v>
       </c>
       <c r="J6" t="n">
+        <v>955.0024194717407</v>
+      </c>
+      <c r="K6" t="n">
         <v>3</v>
       </c>
-      <c r="K6" t="n">
+      <c r="L6" t="n">
         <v>2</v>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="M6" t="inlineStr">
         <is>
           <t>Rx1Tx1, Rx2Tx2</t>
         </is>
@@ -18729,12 +18900,15 @@
         <v>1325.000415086746</v>
       </c>
       <c r="J7" t="n">
+        <v>665.0004150867462</v>
+      </c>
+      <c r="K7" t="n">
         <v>3</v>
       </c>
-      <c r="K7" t="n">
+      <c r="L7" t="n">
         <v>2</v>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="M7" t="inlineStr">
         <is>
           <t>Rx1Tx1, Rx2Tx2</t>
         </is>
@@ -18779,12 +18953,15 @@
         <v>870.0022101402282</v>
       </c>
       <c r="J8" t="n">
-        <v>2</v>
+        <v>660.0022101402282</v>
       </c>
       <c r="K8" t="n">
         <v>2</v>
       </c>
-      <c r="L8" t="inlineStr">
+      <c r="L8" t="n">
+        <v>2</v>
+      </c>
+      <c r="M8" t="inlineStr">
         <is>
           <t>Rx1Tx1, Rx2Tx2</t>
         </is>
@@ -18829,12 +19006,15 @@
         <v>1005.002333641052</v>
       </c>
       <c r="J9" t="n">
+        <v>795.0023336410522</v>
+      </c>
+      <c r="K9" t="n">
         <v>4</v>
       </c>
-      <c r="K9" t="n">
+      <c r="L9" t="n">
         <v>2</v>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="M9" t="inlineStr">
         <is>
           <t>Rx1Tx1, Rx2Tx2</t>
         </is>
@@ -18879,12 +19059,15 @@
         <v>701.0005948543549</v>
       </c>
       <c r="J10" t="n">
-        <v>2</v>
+        <v>546.0005948543549</v>
       </c>
       <c r="K10" t="n">
         <v>2</v>
       </c>
-      <c r="L10" t="inlineStr">
+      <c r="L10" t="n">
+        <v>2</v>
+      </c>
+      <c r="M10" t="inlineStr">
         <is>
           <t>Rx1Tx1, Rx2Tx2</t>
         </is>
@@ -18929,12 +19112,15 @@
         <v>992.9999549388883</v>
       </c>
       <c r="J11" t="n">
+        <v>837.9999549388883</v>
+      </c>
+      <c r="K11" t="n">
         <v>4</v>
       </c>
-      <c r="K11" t="n">
+      <c r="L11" t="n">
         <v>2</v>
       </c>
-      <c r="L11" t="inlineStr">
+      <c r="M11" t="inlineStr">
         <is>
           <t>Rx1Tx1, Rx2Tx2</t>
         </is>
@@ -18979,12 +19165,15 @@
         <v>1289.999727010727</v>
       </c>
       <c r="J12" t="n">
+        <v>561.9997270107267</v>
+      </c>
+      <c r="K12" t="n">
         <v>2</v>
       </c>
-      <c r="K12" t="n">
+      <c r="L12" t="n">
         <v>1</v>
       </c>
-      <c r="L12" t="inlineStr">
+      <c r="M12" t="inlineStr">
         <is>
           <t>Rx1Tx1</t>
         </is>
@@ -19022,13 +19211,13 @@
       <c r="G13" t="n">
         <v>1</v>
       </c>
-      <c r="J13" t="n">
+      <c r="K13" t="n">
         <v>3</v>
       </c>
-      <c r="K13" t="n">
+      <c r="L13" t="n">
         <v>1</v>
       </c>
-      <c r="L13" t="inlineStr">
+      <c r="M13" t="inlineStr">
         <is>
           <t>Rx1Tx1</t>
         </is>
@@ -19066,13 +19255,13 @@
       <c r="G14" t="n">
         <v>1</v>
       </c>
-      <c r="J14" t="n">
+      <c r="K14" t="n">
         <v>2</v>
       </c>
-      <c r="K14" t="n">
+      <c r="L14" t="n">
         <v>1</v>
       </c>
-      <c r="L14" t="inlineStr">
+      <c r="M14" t="inlineStr">
         <is>
           <t>Rx2Tx2</t>
         </is>
@@ -19117,12 +19306,15 @@
         <v>1217.999654054641</v>
       </c>
       <c r="J15" t="n">
+        <v>811.9996540546415</v>
+      </c>
+      <c r="K15" t="n">
         <v>2</v>
       </c>
-      <c r="K15" t="n">
+      <c r="L15" t="n">
         <v>1</v>
       </c>
-      <c r="L15" t="inlineStr">
+      <c r="M15" t="inlineStr">
         <is>
           <t>Rx2Tx2</t>
         </is>
@@ -19160,13 +19352,13 @@
       <c r="G16" t="n">
         <v>1</v>
       </c>
-      <c r="J16" t="n">
+      <c r="K16" t="n">
         <v>3</v>
       </c>
-      <c r="K16" t="n">
+      <c r="L16" t="n">
         <v>1</v>
       </c>
-      <c r="L16" t="inlineStr">
+      <c r="M16" t="inlineStr">
         <is>
           <t>Rx2Tx2</t>
         </is>
@@ -19211,12 +19403,15 @@
         <v>955.9683995246888</v>
       </c>
       <c r="J17" t="n">
+        <v>738.9683995246888</v>
+      </c>
+      <c r="K17" t="n">
         <v>2</v>
       </c>
-      <c r="K17" t="n">
+      <c r="L17" t="n">
         <v>1</v>
       </c>
-      <c r="L17" t="inlineStr">
+      <c r="M17" t="inlineStr">
         <is>
           <t>Rx2Tx2</t>
         </is>
@@ -19261,12 +19456,15 @@
         <v>1413.9799451828</v>
       </c>
       <c r="J18" t="n">
-        <v>2</v>
+        <v>1251.9799451828</v>
       </c>
       <c r="K18" t="n">
         <v>2</v>
       </c>
-      <c r="L18" t="inlineStr">
+      <c r="L18" t="n">
+        <v>2</v>
+      </c>
+      <c r="M18" t="inlineStr">
         <is>
           <t>Rx1Tx1, Rx2Tx2</t>
         </is>
@@ -19311,12 +19509,15 @@
         <v>1049.979978322983</v>
       </c>
       <c r="J19" t="n">
+        <v>887.9799783229828</v>
+      </c>
+      <c r="K19" t="n">
         <v>1</v>
       </c>
-      <c r="K19" t="n">
+      <c r="L19" t="n">
         <v>2</v>
       </c>
-      <c r="L19" t="inlineStr">
+      <c r="M19" t="inlineStr">
         <is>
           <t>Rx1Tx1, Rx2Tx2</t>
         </is>
@@ -19361,12 +19562,15 @@
         <v>1363.962645530701</v>
       </c>
       <c r="J20" t="n">
-        <v>2</v>
+        <v>1135.962645530701</v>
       </c>
       <c r="K20" t="n">
         <v>2</v>
       </c>
-      <c r="L20" t="inlineStr">
+      <c r="L20" t="n">
+        <v>2</v>
+      </c>
+      <c r="M20" t="inlineStr">
         <is>
           <t>Rx1Tx1, Rx2Tx2</t>
         </is>
@@ -19411,12 +19615,15 @@
         <v>955.9626643657683</v>
       </c>
       <c r="J21" t="n">
+        <v>727.9626643657683</v>
+      </c>
+      <c r="K21" t="n">
         <v>1</v>
       </c>
-      <c r="K21" t="n">
+      <c r="L21" t="n">
         <v>2</v>
       </c>
-      <c r="L21" t="inlineStr">
+      <c r="M21" t="inlineStr">
         <is>
           <t>Rx1Tx1, Rx2Tx2</t>
         </is>
@@ -19454,13 +19661,13 @@
       <c r="G22" t="n">
         <v>1</v>
       </c>
-      <c r="J22" t="n">
+      <c r="K22" t="n">
         <v>5</v>
       </c>
-      <c r="K22" t="n">
+      <c r="L22" t="n">
         <v>1</v>
       </c>
-      <c r="L22" t="inlineStr">
+      <c r="M22" t="inlineStr">
         <is>
           <t>Rx2Tx2</t>
         </is>
@@ -19505,12 +19712,15 @@
         <v>1361.965634346008</v>
       </c>
       <c r="J23" t="n">
+        <v>701.9656343460083</v>
+      </c>
+      <c r="K23" t="n">
         <v>3</v>
       </c>
-      <c r="K23" t="n">
+      <c r="L23" t="n">
         <v>1</v>
       </c>
-      <c r="L23" t="inlineStr">
+      <c r="M23" t="inlineStr">
         <is>
           <t>Rx2Tx2</t>
         </is>
@@ -19548,13 +19758,13 @@
       <c r="G24" t="n">
         <v>1</v>
       </c>
-      <c r="J24" t="n">
+      <c r="K24" t="n">
         <v>3</v>
       </c>
-      <c r="K24" t="n">
+      <c r="L24" t="n">
         <v>1</v>
       </c>
-      <c r="L24" t="inlineStr">
+      <c r="M24" t="inlineStr">
         <is>
           <t>Rx2Tx2</t>
         </is>
@@ -19599,19 +19809,22 @@
         <v>1349.999961853027</v>
       </c>
       <c r="J25" t="n">
+        <v>704.9999618530271</v>
+      </c>
+      <c r="K25" t="n">
         <v>3</v>
       </c>
-      <c r="K25" t="n">
+      <c r="L25" t="n">
         <v>1</v>
       </c>
-      <c r="L25" t="inlineStr">
+      <c r="M25" t="inlineStr">
         <is>
           <t>Rx2Tx2</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L25"/>
+  <autoFilter ref="A1:M25"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Restore 10 percent detachment threshold
</commit_message>
<xml_diff>
--- a/outputs/lab_trials/lab_trials_repeatability_report.xlsx
+++ b/outputs/lab_trials/lab_trials_repeatability_report.xlsx
@@ -1740,7 +1740,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>A time is reported only if a positive change point reaches the pre-deposition minus 15% threshold. Otherwise the status is partial.</t>
+          <t>A time is reported only if a positive change point reaches the pre-deposition minus 10% threshold. Otherwise the status is partial.</t>
         </is>
       </c>
     </row>
@@ -1952,7 +1952,7 @@
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>threshold_15pct_lower</t>
+          <t>threshold_10pct_lower</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
@@ -2031,7 +2031,7 @@
         <v>0.5999351032931708</v>
       </c>
       <c r="M2" t="n">
-        <v>0.5099448377991952</v>
+        <v>0.5399415929638537</v>
       </c>
       <c r="N2" t="n">
         <v>0.7190809296697804</v>
@@ -2049,7 +2049,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 15%-below-pre-deposition-reference threshold</t>
+          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 10%-below-pre-deposition-reference threshold</t>
         </is>
       </c>
     </row>
@@ -2103,7 +2103,7 @@
         <v>0.6320859822554428</v>
       </c>
       <c r="M3" t="n">
-        <v>0.5372730849171263</v>
+        <v>0.5688773840298985</v>
       </c>
       <c r="N3" t="n">
         <v>0.5741389473170442</v>
@@ -2121,7 +2121,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 15%-below-pre-deposition-reference threshold</t>
+          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 10%-below-pre-deposition-reference threshold</t>
         </is>
       </c>
     </row>
@@ -2175,7 +2175,7 @@
         <v>0.5987148042124908</v>
       </c>
       <c r="M4" t="n">
-        <v>0.5089075835806172</v>
+        <v>0.5388433237912417</v>
       </c>
       <c r="N4" t="n">
         <v>0.700974947831748</v>
@@ -2193,7 +2193,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 15%-below-pre-deposition-reference threshold</t>
+          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 10%-below-pre-deposition-reference threshold</t>
         </is>
       </c>
     </row>
@@ -2236,7 +2236,7 @@
         <v>3140</v>
       </c>
       <c r="J5" t="n">
-        <v>1880.000734806061</v>
+        <v>2000.000344991684</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -2247,25 +2247,25 @@
         <v>0.6368147672906723</v>
       </c>
       <c r="M5" t="n">
-        <v>0.5412925521970715</v>
+        <v>0.5731332905616051</v>
       </c>
       <c r="N5" t="n">
-        <v>0.5454090153670035</v>
+        <v>0.8339975784746477</v>
       </c>
       <c r="O5" t="n">
         <v>3</v>
       </c>
       <c r="P5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>3 positive upward change points from detachment onset 1630.0s to cooling-window end 3140.0s. First passing point at 1880.0s.</t>
+          <t>3 positive upward change points from detachment onset 1630.0s to cooling-window end 3140.0s. First passing point at 2000.0s.</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 15%-below-pre-deposition-reference threshold</t>
+          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 10%-below-pre-deposition-reference threshold</t>
         </is>
       </c>
     </row>
@@ -2319,7 +2319,7 @@
         <v>0.6009845186289722</v>
       </c>
       <c r="M6" t="n">
-        <v>0.5108368408346263</v>
+        <v>0.540886066766075</v>
       </c>
       <c r="N6" t="n">
         <v>0.592980817588733</v>
@@ -2337,7 +2337,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 15%-below-pre-deposition-reference threshold</t>
+          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 10%-below-pre-deposition-reference threshold</t>
         </is>
       </c>
     </row>
@@ -2391,7 +2391,7 @@
         <v>0.6420872673309568</v>
       </c>
       <c r="M7" t="n">
-        <v>0.5457741772313133</v>
+        <v>0.5778785405978611</v>
       </c>
       <c r="N7" t="n">
         <v>0.8325951321135664</v>
@@ -2409,7 +2409,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 15%-below-pre-deposition-reference threshold</t>
+          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 10%-below-pre-deposition-reference threshold</t>
         </is>
       </c>
     </row>
@@ -2463,7 +2463,7 @@
         <v>0.7328215931830352</v>
       </c>
       <c r="M8" t="n">
-        <v>0.6228983542055799</v>
+        <v>0.6595394338647317</v>
       </c>
       <c r="N8" t="n">
         <v>0.821605322397148</v>
@@ -2481,7 +2481,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 15%-below-pre-deposition-reference threshold</t>
+          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 10%-below-pre-deposition-reference threshold</t>
         </is>
       </c>
     </row>
@@ -2523,19 +2523,16 @@
       <c r="I9" t="n">
         <v>2195</v>
       </c>
-      <c r="J9" t="n">
-        <v>1005.002333641052</v>
-      </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>full_detachment_for_channel</t>
+          <t>partial_detachment_no_change_point_met_threshold</t>
         </is>
       </c>
       <c r="L9" t="n">
         <v>0.6514162486792798</v>
       </c>
       <c r="M9" t="n">
-        <v>0.5537038113773879</v>
+        <v>0.5862746238113519</v>
       </c>
       <c r="N9" t="n">
         <v>0.5637620750490631</v>
@@ -2548,12 +2545,12 @@
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>4 positive upward change points from detachment onset 595.0s to cooling-window end 2195.0s. First passing point at 1005.0s.</t>
+          <t>4 positive upward change points from detachment onset 595.0s to cooling-window end 2195.0s. No change point reached the pre-deposition -10% threshold.</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 15%-below-pre-deposition-reference threshold</t>
+          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 10%-below-pre-deposition-reference threshold</t>
         </is>
       </c>
     </row>
@@ -2607,7 +2604,7 @@
         <v>0.7407382036638537</v>
       </c>
       <c r="M10" t="n">
-        <v>0.6296274731142756</v>
+        <v>0.6666643832974684</v>
       </c>
       <c r="N10" t="n">
         <v>0.9000121704076206</v>
@@ -2625,7 +2622,7 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 15%-below-pre-deposition-reference threshold</t>
+          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 10%-below-pre-deposition-reference threshold</t>
         </is>
       </c>
     </row>
@@ -2679,7 +2676,7 @@
         <v>0.6669369645234606</v>
       </c>
       <c r="M11" t="n">
-        <v>0.5668964198449415</v>
+        <v>0.6002432680711146</v>
       </c>
       <c r="N11" t="n">
         <v>0.699081120081692</v>
@@ -2697,7 +2694,7 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 15%-below-pre-deposition-reference threshold</t>
+          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 10%-below-pre-deposition-reference threshold</t>
         </is>
       </c>
     </row>
@@ -2751,7 +2748,7 @@
         <v>0.7293372337684932</v>
       </c>
       <c r="M12" t="n">
-        <v>0.6199366487032193</v>
+        <v>0.6564035103916439</v>
       </c>
       <c r="N12" t="n">
         <v>0.856245613560319</v>
@@ -2769,7 +2766,7 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 15%-below-pre-deposition-reference threshold</t>
+          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 10%-below-pre-deposition-reference threshold</t>
         </is>
       </c>
     </row>
@@ -2820,7 +2817,7 @@
         <v>0.6557684022430149</v>
       </c>
       <c r="M13" t="n">
-        <v>0.5574031419065627</v>
+        <v>0.5901915620187135</v>
       </c>
       <c r="N13" t="n">
         <v>0.485939799054226</v>
@@ -2833,12 +2830,12 @@
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>3 positive upward change points from detachment onset 1064.0s to cooling-window end 2694.0s. No change point reached the pre-deposition -15% threshold.</t>
+          <t>3 positive upward change points from detachment onset 1064.0s to cooling-window end 2694.0s. No change point reached the pre-deposition -10% threshold.</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 15%-below-pre-deposition-reference threshold</t>
+          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 10%-below-pre-deposition-reference threshold</t>
         </is>
       </c>
     </row>
@@ -2889,7 +2886,7 @@
         <v>0.5923920642654367</v>
       </c>
       <c r="M14" t="n">
-        <v>0.5035332546256212</v>
+        <v>0.533152857838893</v>
       </c>
       <c r="N14" t="n">
         <v>0.2876314729136664</v>
@@ -2902,12 +2899,12 @@
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>2 positive upward change points from detachment onset 1094.0s to cooling-window end 2261.0s. No change point reached the pre-deposition -15% threshold.</t>
+          <t>2 positive upward change points from detachment onset 1094.0s to cooling-window end 2261.0s. No change point reached the pre-deposition -10% threshold.</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 15%-below-pre-deposition-reference threshold</t>
+          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 10%-below-pre-deposition-reference threshold</t>
         </is>
       </c>
     </row>
@@ -2961,7 +2958,7 @@
         <v>0.5936340750157071</v>
       </c>
       <c r="M15" t="n">
-        <v>0.5045889637633511</v>
+        <v>0.5342706675141364</v>
       </c>
       <c r="N15" t="n">
         <v>0.6549491860507034</v>
@@ -2979,7 +2976,7 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 15%-below-pre-deposition-reference threshold</t>
+          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 10%-below-pre-deposition-reference threshold</t>
         </is>
       </c>
     </row>
@@ -3030,7 +3027,7 @@
         <v>0.5855064536151028</v>
       </c>
       <c r="M16" t="n">
-        <v>0.4976804855728374</v>
+        <v>0.5269558082535926</v>
       </c>
       <c r="N16" t="n">
         <v>0.4375577006045251</v>
@@ -3043,12 +3040,12 @@
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>3 positive upward change points from detachment onset 783.0s to cooling-window end 2072.0s. No change point reached the pre-deposition -15% threshold.</t>
+          <t>3 positive upward change points from detachment onset 783.0s to cooling-window end 2072.0s. No change point reached the pre-deposition -10% threshold.</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 15%-below-pre-deposition-reference threshold</t>
+          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 10%-below-pre-deposition-reference threshold</t>
         </is>
       </c>
     </row>
@@ -3102,7 +3099,7 @@
         <v>0.6034922114924255</v>
       </c>
       <c r="M17" t="n">
-        <v>0.5129683797685617</v>
+        <v>0.5431429903431829</v>
       </c>
       <c r="N17" t="n">
         <v>0.7775187872829324</v>
@@ -3120,7 +3117,7 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 15%-below-pre-deposition-reference threshold</t>
+          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 10%-below-pre-deposition-reference threshold</t>
         </is>
       </c>
     </row>
@@ -3162,19 +3159,16 @@
       <c r="I18" t="n">
         <v>2017</v>
       </c>
-      <c r="J18" t="n">
-        <v>1413.9799451828</v>
-      </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>full_detachment_for_channel</t>
+          <t>partial_detachment_no_change_point_met_threshold</t>
         </is>
       </c>
       <c r="L18" t="n">
         <v>0.6090918111618937</v>
       </c>
       <c r="M18" t="n">
-        <v>0.5177280394876096</v>
+        <v>0.5481826300457043</v>
       </c>
       <c r="N18" t="n">
         <v>0.5421488160143766</v>
@@ -3187,12 +3181,12 @@
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>2 positive upward change points from detachment onset 1000.0s to cooling-window end 2017.0s. First passing point at 1414.0s.</t>
+          <t>2 positive upward change points from detachment onset 1000.0s to cooling-window end 2017.0s. No change point reached the pre-deposition -10% threshold.</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 15%-below-pre-deposition-reference threshold</t>
+          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 10%-below-pre-deposition-reference threshold</t>
         </is>
       </c>
     </row>
@@ -3246,7 +3240,7 @@
         <v>0.6091249232898795</v>
       </c>
       <c r="M19" t="n">
-        <v>0.5177561847963976</v>
+        <v>0.5482124309608916</v>
       </c>
       <c r="N19" t="n">
         <v>0.7454181265800934</v>
@@ -3264,7 +3258,7 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 15%-below-pre-deposition-reference threshold</t>
+          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 10%-below-pre-deposition-reference threshold</t>
         </is>
       </c>
     </row>
@@ -3318,7 +3312,7 @@
         <v>0.6207563871985903</v>
       </c>
       <c r="M20" t="n">
-        <v>0.5276429291188017</v>
+        <v>0.5586807484787313</v>
       </c>
       <c r="N20" t="n">
         <v>0.6579884605851972</v>
@@ -3336,7 +3330,7 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 15%-below-pre-deposition-reference threshold</t>
+          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 10%-below-pre-deposition-reference threshold</t>
         </is>
       </c>
     </row>
@@ -3390,7 +3384,7 @@
         <v>0.609385090085468</v>
       </c>
       <c r="M21" t="n">
-        <v>0.5179773265726478</v>
+        <v>0.5484465810769212</v>
       </c>
       <c r="N21" t="n">
         <v>0.8044727888986035</v>
@@ -3408,7 +3402,7 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 15%-below-pre-deposition-reference threshold</t>
+          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 10%-below-pre-deposition-reference threshold</t>
         </is>
       </c>
     </row>
@@ -3459,7 +3453,7 @@
         <v>0.6199542903035502</v>
       </c>
       <c r="M22" t="n">
-        <v>0.5269611467580176</v>
+        <v>0.5579588612731952</v>
       </c>
       <c r="N22" t="n">
         <v>0.4578294486704634</v>
@@ -3472,12 +3466,12 @@
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>5 positive upward change points from detachment onset 1228.0s to cooling-window end 2515.0s. No change point reached the pre-deposition -15% threshold.</t>
+          <t>5 positive upward change points from detachment onset 1228.0s to cooling-window end 2515.0s. No change point reached the pre-deposition -10% threshold.</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 15%-below-pre-deposition-reference threshold</t>
+          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 10%-below-pre-deposition-reference threshold</t>
         </is>
       </c>
     </row>
@@ -3531,7 +3525,7 @@
         <v>0.6023667048574612</v>
       </c>
       <c r="M23" t="n">
-        <v>0.512011699128842</v>
+        <v>0.5421300343717151</v>
       </c>
       <c r="N23" t="n">
         <v>0.7621613005628776</v>
@@ -3549,7 +3543,7 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 15%-below-pre-deposition-reference threshold</t>
+          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 10%-below-pre-deposition-reference threshold</t>
         </is>
       </c>
     </row>
@@ -3600,7 +3594,7 @@
         <v>0.6274948017835749</v>
       </c>
       <c r="M24" t="n">
-        <v>0.5333705815160387</v>
+        <v>0.5647453216052174</v>
       </c>
       <c r="N24" t="n">
         <v>0.4457565432800725</v>
@@ -3613,12 +3607,12 @@
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>3 positive upward change points from detachment onset 1217.0s to cooling-window end 2500.0s. No change point reached the pre-deposition -15% threshold.</t>
+          <t>3 positive upward change points from detachment onset 1217.0s to cooling-window end 2500.0s. No change point reached the pre-deposition -10% threshold.</t>
         </is>
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 15%-below-pre-deposition-reference threshold</t>
+          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 10%-below-pre-deposition-reference threshold</t>
         </is>
       </c>
     </row>
@@ -3672,7 +3666,7 @@
         <v>0.6077120963216972</v>
       </c>
       <c r="M25" t="n">
-        <v>0.5165552818734427</v>
+        <v>0.5469408866895275</v>
       </c>
       <c r="N25" t="n">
         <v>0.7769129392553277</v>
@@ -3690,7 +3684,7 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 15%-below-pre-deposition-reference threshold</t>
+          <t>positive/upward local mean-shift change points; full detachment per channel if US at change point &gt;= 10%-below-pre-deposition-reference threshold</t>
         </is>
       </c>
     </row>
@@ -3775,7 +3769,7 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>threshold_15pct_lower</t>
+          <t>threshold_10pct_lower</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
@@ -3848,7 +3842,7 @@
         <v>0.5999351032931708</v>
       </c>
       <c r="J2" t="n">
-        <v>0.5099448377991952</v>
+        <v>0.5399415929638537</v>
       </c>
       <c r="K2" t="n">
         <v>0.7190809296697804</v>
@@ -3914,7 +3908,7 @@
         <v>0.6320859822554428</v>
       </c>
       <c r="J3" t="n">
-        <v>0.5372730849171263</v>
+        <v>0.5688773840298985</v>
       </c>
       <c r="K3" t="n">
         <v>0.5741389473170442</v>
@@ -3980,7 +3974,7 @@
         <v>0.5987148042124908</v>
       </c>
       <c r="J4" t="n">
-        <v>0.5089075835806172</v>
+        <v>0.5388433237912417</v>
       </c>
       <c r="K4" t="n">
         <v>0.700974947831748</v>
@@ -4040,26 +4034,26 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>1880.000734806061</v>
+        <v>2000.000344991684</v>
       </c>
       <c r="I5" t="n">
         <v>0.6368147672906723</v>
       </c>
       <c r="J5" t="n">
-        <v>0.5412925521970715</v>
+        <v>0.5731332905616051</v>
       </c>
       <c r="K5" t="n">
-        <v>0.5454090153670035</v>
+        <v>0.8339975784746477</v>
       </c>
       <c r="L5" t="n">
         <v>3</v>
       </c>
       <c r="M5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>3 positive upward change points from detachment onset 1630.0s to cooling-window end 3140.0s. First passing point at 1880.0s.</t>
+          <t>3 positive upward change points from detachment onset 1630.0s to cooling-window end 3140.0s. First passing point at 2000.0s.</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -4069,7 +4063,7 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>1 change points before full detachment offset</t>
+          <t>2 change points before full detachment offset</t>
         </is>
       </c>
     </row>
@@ -4112,7 +4106,7 @@
         <v>0.6009845186289722</v>
       </c>
       <c r="J6" t="n">
-        <v>0.5108368408346263</v>
+        <v>0.540886066766075</v>
       </c>
       <c r="K6" t="n">
         <v>0.592980817588733</v>
@@ -4178,7 +4172,7 @@
         <v>0.6420872673309568</v>
       </c>
       <c r="J7" t="n">
-        <v>0.5457741772313133</v>
+        <v>0.5778785405978611</v>
       </c>
       <c r="K7" t="n">
         <v>0.8325951321135664</v>
@@ -4244,7 +4238,7 @@
         <v>0.7328215931830352</v>
       </c>
       <c r="J8" t="n">
-        <v>0.6228983542055799</v>
+        <v>0.6595394338647317</v>
       </c>
       <c r="K8" t="n">
         <v>0.821605322397148</v>
@@ -4300,17 +4294,14 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>full_detachment_for_channel</t>
-        </is>
-      </c>
-      <c r="H9" t="n">
-        <v>1005.002333641052</v>
+          <t>partial_detachment_no_change_point_met_threshold</t>
+        </is>
       </c>
       <c r="I9" t="n">
         <v>0.6514162486792798</v>
       </c>
       <c r="J9" t="n">
-        <v>0.5537038113773879</v>
+        <v>0.5862746238113519</v>
       </c>
       <c r="K9" t="n">
         <v>0.5637620750490631</v>
@@ -4323,7 +4314,7 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>4 positive upward change points from detachment onset 595.0s to cooling-window end 2195.0s. First passing point at 1005.0s.</t>
+          <t>4 positive upward change points from detachment onset 595.0s to cooling-window end 2195.0s. No change point reached the pre-deposition -10% threshold.</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
@@ -4333,7 +4324,7 @@
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>4 change points before full detachment offset</t>
+          <t>4 change points checked; no full detachment offset</t>
         </is>
       </c>
     </row>
@@ -4376,7 +4367,7 @@
         <v>0.7407382036638537</v>
       </c>
       <c r="J10" t="n">
-        <v>0.6296274731142756</v>
+        <v>0.6666643832974684</v>
       </c>
       <c r="K10" t="n">
         <v>0.9000121704076206</v>
@@ -4442,7 +4433,7 @@
         <v>0.6669369645234606</v>
       </c>
       <c r="J11" t="n">
-        <v>0.5668964198449415</v>
+        <v>0.6002432680711146</v>
       </c>
       <c r="K11" t="n">
         <v>0.699081120081692</v>
@@ -4508,7 +4499,7 @@
         <v>0.7293372337684932</v>
       </c>
       <c r="J12" t="n">
-        <v>0.6199366487032193</v>
+        <v>0.6564035103916439</v>
       </c>
       <c r="K12" t="n">
         <v>0.856245613560319</v>
@@ -4571,7 +4562,7 @@
         <v>0.6557684022430149</v>
       </c>
       <c r="J13" t="n">
-        <v>0.5574031419065627</v>
+        <v>0.5901915620187135</v>
       </c>
       <c r="K13" t="n">
         <v>0.485939799054226</v>
@@ -4584,7 +4575,7 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>3 positive upward change points from detachment onset 1064.0s to cooling-window end 2694.0s. No change point reached the pre-deposition -15% threshold.</t>
+          <t>3 positive upward change points from detachment onset 1064.0s to cooling-window end 2694.0s. No change point reached the pre-deposition -10% threshold.</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
@@ -4634,7 +4625,7 @@
         <v>0.5923920642654367</v>
       </c>
       <c r="J14" t="n">
-        <v>0.5035332546256212</v>
+        <v>0.533152857838893</v>
       </c>
       <c r="K14" t="n">
         <v>0.2876314729136664</v>
@@ -4647,7 +4638,7 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>2 positive upward change points from detachment onset 1094.0s to cooling-window end 2261.0s. No change point reached the pre-deposition -15% threshold.</t>
+          <t>2 positive upward change points from detachment onset 1094.0s to cooling-window end 2261.0s. No change point reached the pre-deposition -10% threshold.</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
@@ -4700,7 +4691,7 @@
         <v>0.5936340750157071</v>
       </c>
       <c r="J15" t="n">
-        <v>0.5045889637633511</v>
+        <v>0.5342706675141364</v>
       </c>
       <c r="K15" t="n">
         <v>0.6549491860507034</v>
@@ -4763,7 +4754,7 @@
         <v>0.5855064536151028</v>
       </c>
       <c r="J16" t="n">
-        <v>0.4976804855728374</v>
+        <v>0.5269558082535926</v>
       </c>
       <c r="K16" t="n">
         <v>0.4375577006045251</v>
@@ -4776,7 +4767,7 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>3 positive upward change points from detachment onset 783.0s to cooling-window end 2072.0s. No change point reached the pre-deposition -15% threshold.</t>
+          <t>3 positive upward change points from detachment onset 783.0s to cooling-window end 2072.0s. No change point reached the pre-deposition -10% threshold.</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
@@ -4829,7 +4820,7 @@
         <v>0.6034922114924255</v>
       </c>
       <c r="J17" t="n">
-        <v>0.5129683797685617</v>
+        <v>0.5431429903431829</v>
       </c>
       <c r="K17" t="n">
         <v>0.7775187872829324</v>
@@ -4885,17 +4876,14 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>full_detachment_for_channel</t>
-        </is>
-      </c>
-      <c r="H18" t="n">
-        <v>1413.9799451828</v>
+          <t>partial_detachment_no_change_point_met_threshold</t>
+        </is>
       </c>
       <c r="I18" t="n">
         <v>0.6090918111618937</v>
       </c>
       <c r="J18" t="n">
-        <v>0.5177280394876096</v>
+        <v>0.5481826300457043</v>
       </c>
       <c r="K18" t="n">
         <v>0.5421488160143766</v>
@@ -4908,7 +4896,7 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>2 positive upward change points from detachment onset 1000.0s to cooling-window end 2017.0s. First passing point at 1414.0s.</t>
+          <t>2 positive upward change points from detachment onset 1000.0s to cooling-window end 2017.0s. No change point reached the pre-deposition -10% threshold.</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
@@ -4918,7 +4906,7 @@
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>2 change points before full detachment offset</t>
+          <t>2 change points checked; no full detachment offset</t>
         </is>
       </c>
     </row>
@@ -4961,7 +4949,7 @@
         <v>0.6091249232898795</v>
       </c>
       <c r="J19" t="n">
-        <v>0.5177561847963976</v>
+        <v>0.5482124309608916</v>
       </c>
       <c r="K19" t="n">
         <v>0.7454181265800934</v>
@@ -5027,7 +5015,7 @@
         <v>0.6207563871985903</v>
       </c>
       <c r="J20" t="n">
-        <v>0.5276429291188017</v>
+        <v>0.5586807484787313</v>
       </c>
       <c r="K20" t="n">
         <v>0.6579884605851972</v>
@@ -5093,7 +5081,7 @@
         <v>0.609385090085468</v>
       </c>
       <c r="J21" t="n">
-        <v>0.5179773265726478</v>
+        <v>0.5484465810769212</v>
       </c>
       <c r="K21" t="n">
         <v>0.8044727888986035</v>
@@ -5156,7 +5144,7 @@
         <v>0.6199542903035502</v>
       </c>
       <c r="J22" t="n">
-        <v>0.5269611467580176</v>
+        <v>0.5579588612731952</v>
       </c>
       <c r="K22" t="n">
         <v>0.4578294486704634</v>
@@ -5169,7 +5157,7 @@
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>5 positive upward change points from detachment onset 1228.0s to cooling-window end 2515.0s. No change point reached the pre-deposition -15% threshold.</t>
+          <t>5 positive upward change points from detachment onset 1228.0s to cooling-window end 2515.0s. No change point reached the pre-deposition -10% threshold.</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
@@ -5222,7 +5210,7 @@
         <v>0.6023667048574612</v>
       </c>
       <c r="J23" t="n">
-        <v>0.512011699128842</v>
+        <v>0.5421300343717151</v>
       </c>
       <c r="K23" t="n">
         <v>0.7621613005628776</v>
@@ -5285,7 +5273,7 @@
         <v>0.6274948017835749</v>
       </c>
       <c r="J24" t="n">
-        <v>0.5333705815160387</v>
+        <v>0.5647453216052174</v>
       </c>
       <c r="K24" t="n">
         <v>0.4457565432800725</v>
@@ -5298,7 +5286,7 @@
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>3 positive upward change points from detachment onset 1217.0s to cooling-window end 2500.0s. No change point reached the pre-deposition -15% threshold.</t>
+          <t>3 positive upward change points from detachment onset 1217.0s to cooling-window end 2500.0s. No change point reached the pre-deposition -10% threshold.</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
@@ -5351,7 +5339,7 @@
         <v>0.6077120963216972</v>
       </c>
       <c r="J25" t="n">
-        <v>0.5165552818734427</v>
+        <v>0.5469408866895275</v>
       </c>
       <c r="K25" t="n">
         <v>0.7769129392553277</v>
@@ -11410,7 +11398,7 @@
     <col width="20" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
     <col width="21" customWidth="1" min="9" max="9"/>
-    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="21" customWidth="1" min="10" max="10"/>
     <col width="29" customWidth="1" min="11" max="11"/>
     <col width="32" customWidth="1" min="12" max="12"/>
   </cols>
@@ -11602,13 +11590,13 @@
         <v>3</v>
       </c>
       <c r="F4" t="n">
-        <v>1.666666666666667</v>
+        <v>2</v>
       </c>
       <c r="G4" t="n">
-        <v>1.154700538379252</v>
+        <v>1</v>
       </c>
       <c r="H4" t="n">
-        <v>69.2820323027551</v>
+        <v>50</v>
       </c>
       <c r="I4" t="n">
         <v>1</v>
@@ -11623,7 +11611,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2455_a5/a6/a7 Rx2Tx2 change-point count: CV 69.3%; low repeatability / inspect.</t>
+          <t>2455_a5/a6/a7 Rx2Tx2 change-point count: CV 50.0%; low repeatability / inspect.</t>
         </is>
       </c>
     </row>
@@ -11652,19 +11640,19 @@
         <v>3</v>
       </c>
       <c r="F5" t="n">
-        <v>269.9999094804127</v>
+        <v>309.9997795422871</v>
       </c>
       <c r="G5" t="n">
-        <v>62.45066399874025</v>
+        <v>79.37355405818512</v>
       </c>
       <c r="H5" t="n">
-        <v>23.12988330956117</v>
+        <v>25.60439048549638</v>
       </c>
       <c r="I5" t="n">
         <v>219.9985785484312</v>
       </c>
       <c r="J5" t="n">
-        <v>340.0004150867462</v>
+        <v>370.000344991684</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -11673,7 +11661,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2455_a5/a6/a7 Rx2Tx2 duration: CV 23.1%; low repeatability / inspect.</t>
+          <t>2455_a5/a6/a7 Rx2Tx2 duration: CV 25.6%; low repeatability / inspect.</t>
         </is>
       </c>
     </row>
@@ -11702,16 +11690,16 @@
         <v>3</v>
       </c>
       <c r="F6" t="n">
-        <v>-423.3349270820618</v>
+        <v>-383.3350570201874</v>
       </c>
       <c r="G6" t="n">
-        <v>123.9279600163208</v>
+        <v>82.20903539668039</v>
       </c>
       <c r="H6" t="n">
-        <v>29.27421105329629</v>
+        <v>21.44573888851263</v>
       </c>
       <c r="I6" t="n">
-        <v>-535.0001447200775</v>
+        <v>-445.0026321411135</v>
       </c>
       <c r="J6" t="n">
         <v>-290.0020043849945</v>
@@ -11723,7 +11711,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2455_a5/a6/a7 Rx2Tx2 minus Rx1Tx1 offset: CV 29.3%; low repeatability / inspect.</t>
+          <t>2455_a5/a6/a7 Rx2Tx2 minus Rx1Tx1 offset: CV 21.4%; low repeatability / inspect.</t>
         </is>
       </c>
     </row>
@@ -11949,31 +11937,25 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F11" t="n">
-        <v>462.0011442899703</v>
-      </c>
-      <c r="G11" t="n">
-        <v>73.53742324697041</v>
-      </c>
-      <c r="H11" t="n">
-        <v>15.91715175510808</v>
+        <v>513.9999549388883</v>
       </c>
       <c r="I11" t="n">
-        <v>410.0023336410522</v>
+        <v>513.9999549388883</v>
       </c>
       <c r="J11" t="n">
         <v>513.9999549388883</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>inspect</t>
+          <t>not enough repetitions</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2455_a_test/test3/test4 Rx2Tx2 duration: CV 15.9%; inspect.</t>
+          <t>2455_a_test/test3/test4 Rx2Tx2 duration: CV n/a%; not enough repetitions.</t>
         </is>
       </c>
     </row>
@@ -11999,31 +11981,25 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F12" t="n">
-        <v>213.4997417926788</v>
-      </c>
-      <c r="G12" t="n">
-        <v>111.015224829452</v>
-      </c>
-      <c r="H12" t="n">
-        <v>51.99782627243387</v>
+        <v>291.9993600845335</v>
       </c>
       <c r="I12" t="n">
-        <v>135.0001235008241</v>
+        <v>291.9993600845335</v>
       </c>
       <c r="J12" t="n">
         <v>291.9993600845335</v>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>low repeatability / inspect</t>
+          <t>not enough repetitions</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>2455_a_test/test3/test4 Rx2Tx2 minus Rx1Tx1 offset: CV 52.0%; low repeatability / inspect.</t>
+          <t>2455_a_test/test3/test4 Rx2Tx2 minus Rx1Tx1 offset: CV n/a%; not enough repetitions.</t>
         </is>
       </c>
     </row>
@@ -12052,13 +12028,13 @@
         <v>3</v>
       </c>
       <c r="F13" t="n">
-        <v>1.666666666666667</v>
+        <v>1.333333333333333</v>
       </c>
       <c r="G13" t="n">
         <v>0.5773502691896257</v>
       </c>
       <c r="H13" t="n">
-        <v>34.64101615137754</v>
+        <v>43.30127018922193</v>
       </c>
       <c r="I13" t="n">
         <v>1</v>
@@ -12073,7 +12049,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2455_a_test/test3/test4 number of sensors with full detachment: CV 34.6%; low repeatability / inspect.</t>
+          <t>2455_a_test/test3/test4 number of sensors with full detachment: CV 43.3%; low repeatability / inspect.</t>
         </is>
       </c>
     </row>
@@ -12149,31 +12125,25 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F15" t="n">
-        <v>488.9512953567505</v>
-      </c>
-      <c r="G15" t="n">
-        <v>106.0255002054229</v>
-      </c>
-      <c r="H15" t="n">
-        <v>21.68426614517181</v>
+        <v>563.9226455307007</v>
       </c>
       <c r="I15" t="n">
-        <v>413.9799451828003</v>
+        <v>563.9226455307007</v>
       </c>
       <c r="J15" t="n">
         <v>563.9226455307007</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>low repeatability / inspect</t>
+          <t>not enough repetitions</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>2455_b/b2/b3/b4 Rx1Tx1 duration: CV 21.7%; low repeatability / inspect.</t>
+          <t>2455_b/b2/b3/b4 Rx1Tx1 duration: CV n/a%; not enough repetitions.</t>
         </is>
       </c>
     </row>
@@ -12299,31 +12269,25 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F18" t="n">
-        <v>-385.9999740123749</v>
-      </c>
-      <c r="G18" t="n">
-        <v>31.11270848745182</v>
-      </c>
-      <c r="H18" t="n">
-        <v>8.060287715577504</v>
+        <v>-407.9999811649324</v>
       </c>
       <c r="I18" t="n">
         <v>-407.9999811649324</v>
       </c>
       <c r="J18" t="n">
-        <v>-363.9999668598175</v>
+        <v>-407.9999811649324</v>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>moderate repeatability</t>
+          <t>not enough repetitions</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>2455_b/b2/b3/b4 Rx2Tx2 minus Rx1Tx1 offset: CV 8.1%; moderate repeatability.</t>
+          <t>2455_b/b2/b3/b4 Rx2Tx2 minus Rx1Tx1 offset: CV n/a%; not enough repetitions.</t>
         </is>
       </c>
     </row>
@@ -12352,13 +12316,13 @@
         <v>4</v>
       </c>
       <c r="F19" t="n">
-        <v>1.5</v>
+        <v>1.25</v>
       </c>
       <c r="G19" t="n">
-        <v>0.5773502691896257</v>
+        <v>0.5</v>
       </c>
       <c r="H19" t="n">
-        <v>38.49001794597505</v>
+        <v>40</v>
       </c>
       <c r="I19" t="n">
         <v>1</v>
@@ -12373,7 +12337,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>2455_b/b2/b3/b4 number of sensors with full detachment: CV 38.5%; low repeatability / inspect.</t>
+          <t>2455_b/b2/b3/b4 number of sensors with full detachment: CV 40.0%; low repeatability / inspect.</t>
         </is>
       </c>
     </row>
@@ -12952,13 +12916,13 @@
         <v>1630</v>
       </c>
       <c r="J3" t="n">
-        <v>1880.000734806061</v>
+        <v>2000.000344991684</v>
       </c>
       <c r="K3" t="n">
-        <v>595.0007348060608</v>
+        <v>715.000344991684</v>
       </c>
       <c r="L3" t="n">
-        <v>250.0007348060608</v>
+        <v>370.000344991684</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
@@ -12966,10 +12930,10 @@
         </is>
       </c>
       <c r="N3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O3" t="n">
-        <v>0.5454090153670035</v>
+        <v>0.8339975784746477</v>
       </c>
       <c r="P3" t="inlineStr">
         <is>
@@ -12994,22 +12958,22 @@
         </is>
       </c>
       <c r="V3" t="n">
-        <v>1880.000734806061</v>
+        <v>2000.000344991684</v>
       </c>
       <c r="W3" t="n">
-        <v>595.0007348060608</v>
+        <v>715.000344991684</v>
       </c>
       <c r="X3" t="n">
-        <v>250.0007348060608</v>
+        <v>370.000344991684</v>
       </c>
       <c r="Y3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Z3" t="n">
-        <v>-535.0001447200775</v>
+        <v>-415.0005345344543</v>
       </c>
       <c r="AA3" t="n">
-        <v>-405.0001447200775</v>
+        <v>-285.0005345344543</v>
       </c>
       <c r="AB3" t="n">
         <v>2</v>
@@ -13024,7 +12988,7 @@
       </c>
       <c r="AE3" t="inlineStr">
         <is>
-          <t>2455_a6: 2 sensor(s) reached full US detachment (Rx1Tx1, Rx2Tx2). Rx2 minus Rx1 offset = -535.0 s.</t>
+          <t>2455_a6: 2 sensor(s) reached full US detachment (Rx1Tx1, Rx2Tx2). Rx2 minus Rx1 offset = -415.0 s.</t>
         </is>
       </c>
     </row>
@@ -13185,18 +13149,9 @@
       <c r="I5" t="n">
         <v>595</v>
       </c>
-      <c r="J5" t="n">
-        <v>1005.002333641052</v>
-      </c>
-      <c r="K5" t="n">
-        <v>795.0023336410522</v>
-      </c>
-      <c r="L5" t="n">
-        <v>410.0023336410522</v>
-      </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>full_detachment_for_channel</t>
+          <t>partial_detachment_no_change_point_met_threshold</t>
         </is>
       </c>
       <c r="N5" t="n">
@@ -13224,41 +13179,26 @@
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>full_detachment_for_channel</t>
-        </is>
-      </c>
-      <c r="V5" t="n">
-        <v>1005.002333641052</v>
-      </c>
-      <c r="W5" t="n">
-        <v>795.0023336410522</v>
-      </c>
-      <c r="X5" t="n">
-        <v>410.0023336410522</v>
+          <t>partial_detachment_no_change_point_met_threshold</t>
+        </is>
       </c>
       <c r="Y5" t="n">
         <v>4</v>
       </c>
-      <c r="Z5" t="n">
-        <v>135.0001235008241</v>
-      </c>
-      <c r="AA5" t="n">
-        <v>140.0001235008241</v>
-      </c>
       <c r="AB5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AC5" t="inlineStr">
         <is>
-          <t>Rx1Tx1, Rx2Tx2</t>
+          <t>Rx1Tx1</t>
         </is>
       </c>
       <c r="AD5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AE5" t="inlineStr">
         <is>
-          <t>2455_a_test: 2 sensor(s) reached full US detachment (Rx1Tx1, Rx2Tx2). Rx2 minus Rx1 offset = 135.0 s.</t>
+          <t>2455_a_test: 1 sensor(s) reached full US detachment (Rx1Tx1). Rx2 minus Rx1 offset = n/a s.</t>
         </is>
       </c>
     </row>
@@ -13738,17 +13678,8 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>full_detachment_for_channel</t>
-        </is>
-      </c>
-      <c r="Q10" t="n">
-        <v>1413.9799451828</v>
-      </c>
-      <c r="R10" t="n">
-        <v>1251.9799451828</v>
-      </c>
-      <c r="S10" t="n">
-        <v>413.9799451828003</v>
+          <t>partial_detachment_no_change_point_met_threshold</t>
+        </is>
       </c>
       <c r="T10" t="n">
         <v>2</v>
@@ -13770,26 +13701,20 @@
       <c r="Y10" t="n">
         <v>1</v>
       </c>
-      <c r="Z10" t="n">
-        <v>-363.9999668598175</v>
-      </c>
-      <c r="AA10" t="n">
-        <v>-361.9999668598175</v>
-      </c>
       <c r="AB10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AC10" t="inlineStr">
         <is>
-          <t>Rx1Tx1, Rx2Tx2</t>
+          <t>Rx2Tx2</t>
         </is>
       </c>
       <c r="AD10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AE10" t="inlineStr">
         <is>
-          <t>2455_b3: 2 sensor(s) reached full US detachment (Rx1Tx1, Rx2Tx2). Rx2 minus Rx1 offset = -364.0 s.</t>
+          <t>2455_b3: 1 sensor(s) reached full US detachment (Rx2Tx2). Rx2 minus Rx1 offset = n/a s.</t>
         </is>
       </c>
     </row>
@@ -14231,7 +14156,7 @@
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Rx1Tx1 CP count vs Rx2Tx2 CP count: r=0.146, n=12; very weak agreement.</t>
+          <t>Rx1Tx1 CP count vs Rx2Tx2 CP count: r=0.194, n=12; very weak agreement.</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -14262,7 +14187,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -14272,7 +14197,7 @@
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Rx1Tx1 duration vs Rx2Tx2 duration: r=-0.616, n=7; strong agreement.</t>
+          <t>Rx1Tx1 duration vs Rx2Tx2 duration: r=-0.647, n=5; strong agreement.</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -14656,17 +14581,17 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Trials</t>
+          <t>Cooling Configuration</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F11" t="n">
         <v>2</v>
       </c>
       <c r="G11" t="n">
-        <v>0.9138627970170046</v>
+        <v>0.9240306555533012</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
@@ -14675,12 +14600,12 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>MOAN (561.7) vs Marcos (229.3)</t>
+          <t>Cooling S (562.2) vs Marcos Cooling Tunnel (229.3)</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Trials shows a large screened association with Rx1Tx1 detachment duration; largest mean contrast: MOAN (561.7) vs Marcos (229.3).</t>
+          <t>Cooling Configuration shows a large screened association with Rx1Tx1 detachment duration; largest mean contrast: Cooling S (562.2) vs Marcos Cooling Tunnel (229.3).</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -14707,17 +14632,17 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Cooling Configuration</t>
+          <t>Cooling Temperature (°C)</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F12" t="n">
         <v>2</v>
       </c>
       <c r="G12" t="n">
-        <v>0.8385312134352619</v>
+        <v>0.9240306555533012</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
@@ -14726,12 +14651,12 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Cooling S (532.6) vs Marcos Cooling Tunnel (229.3)</t>
+          <t>15 (562.2) vs 15 to 12 to 15 (229.3)</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Cooling Configuration shows a large screened association with Rx1Tx1 detachment duration; largest mean contrast: Cooling S (532.6) vs Marcos Cooling Tunnel (229.3).</t>
+          <t>Cooling Temperature (°C) shows a large screened association with Rx1Tx1 detachment duration; largest mean contrast: 15 (562.2) vs 15 to 12 to 15 (229.3).</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -14758,17 +14683,17 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Cooling Temperature (°C)</t>
+          <t>Trials</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F13" t="n">
         <v>2</v>
       </c>
       <c r="G13" t="n">
-        <v>0.8385312134352619</v>
+        <v>0.9138627970170046</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
@@ -14777,12 +14702,12 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>15 (532.6) vs 15 to 12 to 15 (229.3)</t>
+          <t>MOAN (561.7) vs Marcos (229.3)</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Cooling Temperature (°C) shows a large screened association with Rx1Tx1 detachment duration; largest mean contrast: 15 (532.6) vs 15 to 12 to 15 (229.3).</t>
+          <t>Trials shows a large screened association with Rx1Tx1 detachment duration; largest mean contrast: MOAN (561.7) vs Marcos (229.3).</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -14813,13 +14738,13 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F14" t="n">
         <v>2</v>
       </c>
       <c r="G14" t="n">
-        <v>0.06370525256328548</v>
+        <v>0.11825784013118</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
@@ -14828,12 +14753,12 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Milk (489) vs Dark (395.5)</t>
+          <t>Milk (563.9) vs Dark (395.5)</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Chocolate Recipe shows a small screened association with Rx1Tx1 detachment duration; largest mean contrast: Milk (489) vs Dark (395.5).</t>
+          <t>Chocolate Recipe shows a small screened association with Rx1Tx1 detachment duration; largest mean contrast: Milk (563.9) vs Dark (395.5).</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -14864,13 +14789,13 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F15" t="n">
         <v>2</v>
       </c>
       <c r="G15" t="n">
-        <v>0.06370525256328548</v>
+        <v>0.11825784013118</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
@@ -14879,12 +14804,12 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>AMC (489) vs Stella (395.5)</t>
+          <t>AMC (563.9) vs Stella (395.5)</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Tempering shows a small screened association with Rx1Tx1 detachment duration; largest mean contrast: AMC (489) vs Stella (395.5).</t>
+          <t>Tempering shows a small screened association with Rx1Tx1 detachment duration; largest mean contrast: AMC (563.9) vs Stella (395.5).</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -14915,13 +14840,13 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F16" t="n">
         <v>2</v>
       </c>
       <c r="G16" t="n">
-        <v>0.06370525256328548</v>
+        <v>0.11825784013118</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
@@ -14930,12 +14855,12 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>4.9 (489) vs 0.2-0.4 UT (395.5)</t>
+          <t>4.9 (563.9) vs 0.2-0.4 UT (395.5)</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Tempering Degree shows a small screened association with Rx1Tx1 detachment duration; largest mean contrast: 4.9 (489) vs 0.2-0.4 UT (395.5).</t>
+          <t>Tempering Degree shows a small screened association with Rx1Tx1 detachment duration; largest mean contrast: 4.9 (563.9) vs 0.2-0.4 UT (395.5).</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -14972,7 +14897,7 @@
         <v>3</v>
       </c>
       <c r="G17" t="n">
-        <v>0.6491228070175437</v>
+        <v>0.612121212121212</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
@@ -14981,12 +14906,12 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Marcos (3.667) vs MOAN (1.667)</t>
+          <t>Marcos (3.667) vs MOAN (2)</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Trials shows a large screened association with Rx2Tx2 change-point count; largest mean contrast: Marcos (3.667) vs MOAN (1.667).</t>
+          <t>Trials shows a large screened association with Rx2Tx2 change-point count; largest mean contrast: Marcos (3.667) vs MOAN (2).</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -15023,7 +14948,7 @@
         <v>2</v>
       </c>
       <c r="G18" t="n">
-        <v>0.4848484848484848</v>
+        <v>0.4838709677419353</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
@@ -15032,12 +14957,12 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Marcos Cooling Tunnel (3.667) vs Cooling S (1.889)</t>
+          <t>Marcos Cooling Tunnel (3.667) vs Cooling S (2)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Cooling Configuration shows a large screened association with Rx2Tx2 change-point count; largest mean contrast: Marcos Cooling Tunnel (3.667) vs Cooling S (1.889).</t>
+          <t>Cooling Configuration shows a large screened association with Rx2Tx2 change-point count; largest mean contrast: Marcos Cooling Tunnel (3.667) vs Cooling S (2).</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -15074,7 +14999,7 @@
         <v>2</v>
       </c>
       <c r="G19" t="n">
-        <v>0.4848484848484848</v>
+        <v>0.4838709677419353</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
@@ -15083,12 +15008,12 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>15 to 12 to 15 (3.667) vs 15 (1.889)</t>
+          <t>15 to 12 to 15 (3.667) vs 15 (2)</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>Cooling Temperature (°C) shows a large screened association with Rx2Tx2 change-point count; largest mean contrast: 15 to 12 to 15 (3.667) vs 15 (1.889).</t>
+          <t>Cooling Temperature (°C) shows a large screened association with Rx2Tx2 change-point count; largest mean contrast: 15 to 12 to 15 (3.667) vs 15 (2).</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -15125,7 +15050,7 @@
         <v>2</v>
       </c>
       <c r="G20" t="n">
-        <v>0.4608294930875576</v>
+        <v>0.4285714285714286</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
@@ -15134,12 +15059,12 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>20.0 (3) vs 35.0 (1.571)</t>
+          <t>20.0 (3) vs 35.0 (1.714)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>Cooling Speed (%) shows a large screened association with Rx2Tx2 change-point count; largest mean contrast: 20.0 (3) vs 35.0 (1.571).</t>
+          <t>Cooling Speed (%) shows a large screened association with Rx2Tx2 change-point count; largest mean contrast: 20.0 (3) vs 35.0 (1.714).</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -15176,21 +15101,21 @@
         <v>2</v>
       </c>
       <c r="G21" t="n">
-        <v>0.284090909090909</v>
+        <v>0.3903225806451612</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>moderate</t>
+          <t>large</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Dark (2.75) vs Milk (1.5)</t>
+          <t>Dark (2.875) vs Milk (1.5)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Chocolate Recipe shows a moderate screened association with Rx2Tx2 change-point count; largest mean contrast: Dark (2.75) vs Milk (1.5).</t>
+          <t>Chocolate Recipe shows a large screened association with Rx2Tx2 change-point count; largest mean contrast: Dark (2.875) vs Milk (1.5).</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -15227,21 +15152,21 @@
         <v>2</v>
       </c>
       <c r="G22" t="n">
-        <v>0.284090909090909</v>
+        <v>0.3903225806451612</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>moderate</t>
+          <t>large</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Stella (2.75) vs AMC (1.5)</t>
+          <t>Stella (2.875) vs AMC (1.5)</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Tempering shows a moderate screened association with Rx2Tx2 change-point count; largest mean contrast: Stella (2.75) vs AMC (1.5).</t>
+          <t>Tempering shows a large screened association with Rx2Tx2 change-point count; largest mean contrast: Stella (2.875) vs AMC (1.5).</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -15278,21 +15203,21 @@
         <v>2</v>
       </c>
       <c r="G23" t="n">
-        <v>0.284090909090909</v>
+        <v>0.3903225806451612</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>moderate</t>
+          <t>large</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>0.2-0.4 UT (2.75) vs 4.9 (1.5)</t>
+          <t>0.2-0.4 UT (2.875) vs 4.9 (1.5)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>Tempering Degree shows a moderate screened association with Rx2Tx2 change-point count; largest mean contrast: 0.2-0.4 UT (2.75) vs 4.9 (1.5).</t>
+          <t>Tempering Degree shows a large screened association with Rx2Tx2 change-point count; largest mean contrast: 0.2-0.4 UT (2.875) vs 4.9 (1.5).</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -15323,13 +15248,13 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F24" t="n">
         <v>3</v>
       </c>
       <c r="G24" t="n">
-        <v>0.7750684809411131</v>
+        <v>0.733115176184031</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
@@ -15338,12 +15263,12 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Marcos (462) vs MOAN (270)</t>
+          <t>Marcos (514) vs HASS (301.5)</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Trials shows a large screened association with Rx2Tx2 detachment duration; largest mean contrast: Marcos (462) vs MOAN (270).</t>
+          <t>Trials shows a large screened association with Rx2Tx2 detachment duration; largest mean contrast: Marcos (514) vs HASS (301.5).</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -15370,17 +15295,17 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Cooling Configuration</t>
+          <t>Chocolate Recipe</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F25" t="n">
         <v>2</v>
       </c>
       <c r="G25" t="n">
-        <v>0.5368831484708115</v>
+        <v>0.5232099084803775</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
@@ -15389,12 +15314,12 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Marcos Cooling Tunnel (462) vs Cooling S (225.5)</t>
+          <t>Dark (341.2) vs Milk (154.2)</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>Cooling Configuration shows a large screened association with Rx2Tx2 detachment duration; largest mean contrast: Marcos Cooling Tunnel (462) vs Cooling S (225.5).</t>
+          <t>Chocolate Recipe shows a large screened association with Rx2Tx2 detachment duration; largest mean contrast: Dark (341.2) vs Milk (154.2).</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -15421,17 +15346,17 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Cooling Temperature (°C)</t>
+          <t>Tempering</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F26" t="n">
         <v>2</v>
       </c>
       <c r="G26" t="n">
-        <v>0.5368831484708115</v>
+        <v>0.5232099084803775</v>
       </c>
       <c r="H26" t="inlineStr">
         <is>
@@ -15440,12 +15365,12 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>15 to 12 to 15 (462) vs 15 (225.5)</t>
+          <t>Stella (341.2) vs AMC (154.2)</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Cooling Temperature (°C) shows a large screened association with Rx2Tx2 detachment duration; largest mean contrast: 15 to 12 to 15 (462) vs 15 (225.5).</t>
+          <t>Tempering shows a large screened association with Rx2Tx2 detachment duration; largest mean contrast: Stella (341.2) vs AMC (154.2).</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -15472,17 +15397,17 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Chocolate Recipe</t>
+          <t>Tempering Degree</t>
         </is>
       </c>
       <c r="E27" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F27" t="n">
         <v>2</v>
       </c>
       <c r="G27" t="n">
-        <v>0.4819934221539969</v>
+        <v>0.5232099084803775</v>
       </c>
       <c r="H27" t="inlineStr">
         <is>
@@ -15491,12 +15416,12 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Dark (333.9) vs Milk (154.2)</t>
+          <t>0.2-0.4 UT (341.2) vs 4.9 (154.2)</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>Chocolate Recipe shows a large screened association with Rx2Tx2 detachment duration; largest mean contrast: Dark (333.9) vs Milk (154.2).</t>
+          <t>Tempering Degree shows a large screened association with Rx2Tx2 detachment duration; largest mean contrast: 0.2-0.4 UT (341.2) vs 4.9 (154.2).</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -15523,17 +15448,17 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Tempering</t>
+          <t>Cooling Configuration</t>
         </is>
       </c>
       <c r="E28" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F28" t="n">
         <v>2</v>
       </c>
       <c r="G28" t="n">
-        <v>0.4819934221539969</v>
+        <v>0.4249497844018145</v>
       </c>
       <c r="H28" t="inlineStr">
         <is>
@@ -15542,12 +15467,12 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Stella (333.9) vs AMC (154.2)</t>
+          <t>Marcos Cooling Tunnel (514) vs Cooling S (238.9)</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Tempering shows a large screened association with Rx2Tx2 detachment duration; largest mean contrast: Stella (333.9) vs AMC (154.2).</t>
+          <t>Cooling Configuration shows a large screened association with Rx2Tx2 detachment duration; largest mean contrast: Marcos Cooling Tunnel (514) vs Cooling S (238.9).</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -15574,17 +15499,17 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Tempering Degree</t>
+          <t>Cooling Temperature (°C)</t>
         </is>
       </c>
       <c r="E29" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F29" t="n">
         <v>2</v>
       </c>
       <c r="G29" t="n">
-        <v>0.4819934221539969</v>
+        <v>0.4249497844018145</v>
       </c>
       <c r="H29" t="inlineStr">
         <is>
@@ -15593,12 +15518,12 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>0.2-0.4 UT (333.9) vs 4.9 (154.2)</t>
+          <t>15 to 12 to 15 (514) vs 15 (238.9)</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>Tempering Degree shows a large screened association with Rx2Tx2 detachment duration; largest mean contrast: 0.2-0.4 UT (333.9) vs 4.9 (154.2).</t>
+          <t>Cooling Temperature (°C) shows a large screened association with Rx2Tx2 detachment duration; largest mean contrast: 15 to 12 to 15 (514) vs 15 (238.9).</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -15635,21 +15560,21 @@
         <v>2</v>
       </c>
       <c r="G30" t="n">
-        <v>0.2017474565239897</v>
+        <v>0.1093561675530039</v>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>moderate</t>
+          <t>small</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>20.0 (301.5) vs 35.0 (203.8)</t>
+          <t>20.0 (301.5) vs 35.0 (221)</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Cooling Speed (%) shows a moderate screened association with Rx2Tx2 detachment duration; largest mean contrast: 20.0 (301.5) vs 35.0 (203.8).</t>
+          <t>Cooling Speed (%) shows a small screened association with Rx2Tx2 detachment duration; largest mean contrast: 20.0 (301.5) vs 35.0 (221).</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -15680,13 +15605,13 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F31" t="n">
         <v>2</v>
       </c>
       <c r="G31" t="n">
-        <v>0.923634869212138</v>
+        <v>0.9637563532448646</v>
       </c>
       <c r="H31" t="inlineStr">
         <is>
@@ -15695,12 +15620,12 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Marcos Cooling Tunnel (213.5) vs Cooling S (-408.4)</t>
+          <t>Marcos Cooling Tunnel (292) vs Cooling S (-389.5)</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>Cooling Configuration shows a large screened association with Rx2Tx2 minus Rx1Tx1 offset time; largest mean contrast: Marcos Cooling Tunnel (213.5) vs Cooling S (-408.4).</t>
+          <t>Cooling Configuration shows a large screened association with Rx2Tx2 minus Rx1Tx1 offset time; largest mean contrast: Marcos Cooling Tunnel (292) vs Cooling S (-389.5).</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -15731,13 +15656,13 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F32" t="n">
         <v>2</v>
       </c>
       <c r="G32" t="n">
-        <v>0.923634869212138</v>
+        <v>0.9637563532448646</v>
       </c>
       <c r="H32" t="inlineStr">
         <is>
@@ -15746,12 +15671,12 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>15 to 12 to 15 (213.5) vs 15 (-408.4)</t>
+          <t>15 to 12 to 15 (292) vs 15 (-389.5)</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>Cooling Temperature (°C) shows a large screened association with Rx2Tx2 minus Rx1Tx1 offset time; largest mean contrast: 15 to 12 to 15 (213.5) vs 15 (-408.4).</t>
+          <t>Cooling Temperature (°C) shows a large screened association with Rx2Tx2 minus Rx1Tx1 offset time; largest mean contrast: 15 to 12 to 15 (292) vs 15 (-389.5).</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -15782,13 +15707,13 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F33" t="n">
         <v>2</v>
       </c>
       <c r="G33" t="n">
-        <v>0.9187468631681847</v>
+        <v>0.9619863998010915</v>
       </c>
       <c r="H33" t="inlineStr">
         <is>
@@ -15797,12 +15722,12 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>Marcos (213.5) vs MOAN (-423.3)</t>
+          <t>Marcos (292) vs MOAN (-383.3)</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>Trials shows a large screened association with Rx2Tx2 minus Rx1Tx1 offset time; largest mean contrast: Marcos (213.5) vs MOAN (-423.3).</t>
+          <t>Trials shows a large screened association with Rx2Tx2 minus Rx1Tx1 offset time; largest mean contrast: Marcos (292) vs MOAN (-383.3).</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -15833,13 +15758,13 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F34" t="n">
         <v>2</v>
       </c>
       <c r="G34" t="n">
-        <v>0.1128685611080733</v>
+        <v>0.0776944578631685</v>
       </c>
       <c r="H34" t="inlineStr">
         <is>
@@ -15848,12 +15773,12 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>Dark (-168.6) vs Milk (-386)</t>
+          <t>Dark (-214.5) vs Milk (-408)</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>Chocolate Recipe shows a small screened association with Rx2Tx2 minus Rx1Tx1 offset time; largest mean contrast: Dark (-168.6) vs Milk (-386).</t>
+          <t>Chocolate Recipe shows a small screened association with Rx2Tx2 minus Rx1Tx1 offset time; largest mean contrast: Dark (-214.5) vs Milk (-408).</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -15884,13 +15809,13 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F35" t="n">
         <v>2</v>
       </c>
       <c r="G35" t="n">
-        <v>0.1128685611080733</v>
+        <v>0.0776944578631685</v>
       </c>
       <c r="H35" t="inlineStr">
         <is>
@@ -15899,12 +15824,12 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>Stella (-168.6) vs AMC (-386)</t>
+          <t>Stella (-214.5) vs AMC (-408)</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>Tempering shows a small screened association with Rx2Tx2 minus Rx1Tx1 offset time; largest mean contrast: Stella (-168.6) vs AMC (-386).</t>
+          <t>Tempering shows a small screened association with Rx2Tx2 minus Rx1Tx1 offset time; largest mean contrast: Stella (-214.5) vs AMC (-408).</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -15935,13 +15860,13 @@
         </is>
       </c>
       <c r="E36" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F36" t="n">
         <v>2</v>
       </c>
       <c r="G36" t="n">
-        <v>0.1128685611080733</v>
+        <v>0.0776944578631685</v>
       </c>
       <c r="H36" t="inlineStr">
         <is>
@@ -15950,12 +15875,12 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>0.2-0.4 UT (-168.6) vs 4.9 (-386)</t>
+          <t>0.2-0.4 UT (-214.5) vs 4.9 (-408)</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>Tempering Degree shows a small screened association with Rx2Tx2 minus Rx1Tx1 offset time; largest mean contrast: 0.2-0.4 UT (-168.6) vs 4.9 (-386).</t>
+          <t>Tempering Degree shows a small screened association with Rx2Tx2 minus Rx1Tx1 offset time; largest mean contrast: 0.2-0.4 UT (-214.5) vs 4.9 (-408).</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -15992,7 +15917,7 @@
         <v>3</v>
       </c>
       <c r="G37" t="n">
-        <v>0.6444444444444444</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="H37" t="inlineStr">
         <is>
@@ -16043,21 +15968,21 @@
         <v>2</v>
       </c>
       <c r="G38" t="n">
-        <v>0.3571428571428572</v>
+        <v>0.2285714285714285</v>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>large</t>
+          <t>moderate</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>35.0 (0.7143) vs 20.0 (0)</t>
+          <t>35.0 (0.5714) vs 20.0 (0)</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>Cooling Speed (%) shows a large screened association with both channels full-offset probability; largest mean contrast: 35.0 (0.7143) vs 20.0 (0).</t>
+          <t>Cooling Speed (%) shows a moderate screened association with both channels full-offset probability; largest mean contrast: 35.0 (0.5714) vs 20.0 (0).</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -16094,7 +16019,7 @@
         <v>2</v>
       </c>
       <c r="G39" t="n">
-        <v>0.01428571428571429</v>
+        <v>0.05714285714285714</v>
       </c>
       <c r="H39" t="inlineStr">
         <is>
@@ -16103,12 +16028,12 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>Dark (0.625) vs Milk (0.5)</t>
+          <t>Dark (0.5) vs Milk (0.25)</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>Chocolate Recipe shows a weak screened association with both channels full-offset probability; largest mean contrast: Dark (0.625) vs Milk (0.5).</t>
+          <t>Chocolate Recipe shows a weak screened association with both channels full-offset probability; largest mean contrast: Dark (0.5) vs Milk (0.25).</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -16145,7 +16070,7 @@
         <v>2</v>
       </c>
       <c r="G40" t="n">
-        <v>0.01428571428571429</v>
+        <v>0.05714285714285714</v>
       </c>
       <c r="H40" t="inlineStr">
         <is>
@@ -16154,12 +16079,12 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>Stella (0.625) vs AMC (0.5)</t>
+          <t>Stella (0.5) vs AMC (0.25)</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>Tempering shows a weak screened association with both channels full-offset probability; largest mean contrast: Stella (0.625) vs AMC (0.5).</t>
+          <t>Tempering shows a weak screened association with both channels full-offset probability; largest mean contrast: Stella (0.5) vs AMC (0.25).</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -16196,7 +16121,7 @@
         <v>2</v>
       </c>
       <c r="G41" t="n">
-        <v>0.01428571428571429</v>
+        <v>0.05714285714285714</v>
       </c>
       <c r="H41" t="inlineStr">
         <is>
@@ -16205,12 +16130,12 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>0.2-0.4 UT (0.625) vs 4.9 (0.5)</t>
+          <t>0.2-0.4 UT (0.5) vs 4.9 (0.25)</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>Tempering Degree shows a weak screened association with both channels full-offset probability; largest mean contrast: 0.2-0.4 UT (0.625) vs 4.9 (0.5).</t>
+          <t>Tempering Degree shows a weak screened association with both channels full-offset probability; largest mean contrast: 0.2-0.4 UT (0.5) vs 4.9 (0.25).</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -16247,7 +16172,7 @@
         <v>2</v>
       </c>
       <c r="G42" t="n">
-        <v>0.009523809523809513</v>
+        <v>0.009523809523809523</v>
       </c>
       <c r="H42" t="inlineStr">
         <is>
@@ -16256,12 +16181,12 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>Marcos Cooling Tunnel (0.6667) vs Cooling S (0.5556)</t>
+          <t>Cooling S (0.4444) vs Marcos Cooling Tunnel (0.3333)</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>Cooling Configuration shows a weak screened association with both channels full-offset probability; largest mean contrast: Marcos Cooling Tunnel (0.6667) vs Cooling S (0.5556).</t>
+          <t>Cooling Configuration shows a weak screened association with both channels full-offset probability; largest mean contrast: Cooling S (0.4444) vs Marcos Cooling Tunnel (0.3333).</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -16298,7 +16223,7 @@
         <v>2</v>
       </c>
       <c r="G43" t="n">
-        <v>0.009523809523809513</v>
+        <v>0.009523809523809523</v>
       </c>
       <c r="H43" t="inlineStr">
         <is>
@@ -16307,12 +16232,12 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>15 to 12 to 15 (0.6667) vs 15 (0.5556)</t>
+          <t>15 (0.4444) vs 15 to 12 to 15 (0.3333)</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>Cooling Temperature (°C) shows a weak screened association with both channels full-offset probability; largest mean contrast: 15 to 12 to 15 (0.6667) vs 15 (0.5556).</t>
+          <t>Cooling Temperature (°C) shows a weak screened association with both channels full-offset probability; largest mean contrast: 15 (0.4444) vs 15 to 12 to 15 (0.3333).</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
@@ -16349,7 +16274,7 @@
         <v>3</v>
       </c>
       <c r="G44" t="n">
-        <v>0.6444444444444444</v>
+        <v>0.6666666666666667</v>
       </c>
       <c r="H44" t="inlineStr">
         <is>
@@ -16400,21 +16325,21 @@
         <v>2</v>
       </c>
       <c r="G45" t="n">
-        <v>0.357142857142857</v>
+        <v>0.2285714285714285</v>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>large</t>
+          <t>moderate</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>35.0 (1.714) vs 20.0 (1)</t>
+          <t>35.0 (1.571) vs 20.0 (1)</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>Cooling Speed (%) shows a large screened association with number of sensors with full detachment; largest mean contrast: 35.0 (1.714) vs 20.0 (1).</t>
+          <t>Cooling Speed (%) shows a moderate screened association with number of sensors with full detachment; largest mean contrast: 35.0 (1.571) vs 20.0 (1).</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -16451,7 +16376,7 @@
         <v>2</v>
       </c>
       <c r="G46" t="n">
-        <v>0.01428571428571429</v>
+        <v>0.05714285714285715</v>
       </c>
       <c r="H46" t="inlineStr">
         <is>
@@ -16460,12 +16385,12 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>Dark (1.625) vs Milk (1.5)</t>
+          <t>Dark (1.5) vs Milk (1.25)</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>Chocolate Recipe shows a weak screened association with number of sensors with full detachment; largest mean contrast: Dark (1.625) vs Milk (1.5).</t>
+          <t>Chocolate Recipe shows a weak screened association with number of sensors with full detachment; largest mean contrast: Dark (1.5) vs Milk (1.25).</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
@@ -16502,7 +16427,7 @@
         <v>2</v>
       </c>
       <c r="G47" t="n">
-        <v>0.01428571428571429</v>
+        <v>0.05714285714285715</v>
       </c>
       <c r="H47" t="inlineStr">
         <is>
@@ -16511,12 +16436,12 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>Stella (1.625) vs AMC (1.5)</t>
+          <t>Stella (1.5) vs AMC (1.25)</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>Tempering shows a weak screened association with number of sensors with full detachment; largest mean contrast: Stella (1.625) vs AMC (1.5).</t>
+          <t>Tempering shows a weak screened association with number of sensors with full detachment; largest mean contrast: Stella (1.5) vs AMC (1.25).</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
@@ -16553,7 +16478,7 @@
         <v>2</v>
       </c>
       <c r="G48" t="n">
-        <v>0.01428571428571429</v>
+        <v>0.05714285714285715</v>
       </c>
       <c r="H48" t="inlineStr">
         <is>
@@ -16562,12 +16487,12 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>0.2-0.4 UT (1.625) vs 4.9 (1.5)</t>
+          <t>0.2-0.4 UT (1.5) vs 4.9 (1.25)</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>Tempering Degree shows a weak screened association with number of sensors with full detachment; largest mean contrast: 0.2-0.4 UT (1.625) vs 4.9 (1.5).</t>
+          <t>Tempering Degree shows a weak screened association with number of sensors with full detachment; largest mean contrast: 0.2-0.4 UT (1.5) vs 4.9 (1.25).</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
@@ -16613,12 +16538,12 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>Marcos Cooling Tunnel (1.667) vs Cooling S (1.556)</t>
+          <t>Cooling S (1.444) vs Marcos Cooling Tunnel (1.333)</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>Cooling Configuration shows a weak screened association with number of sensors with full detachment; largest mean contrast: Marcos Cooling Tunnel (1.667) vs Cooling S (1.556).</t>
+          <t>Cooling Configuration shows a weak screened association with number of sensors with full detachment; largest mean contrast: Cooling S (1.444) vs Marcos Cooling Tunnel (1.333).</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
@@ -16664,12 +16589,12 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>15 to 12 to 15 (1.667) vs 15 (1.556)</t>
+          <t>15 (1.444) vs 15 to 12 to 15 (1.333)</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>Cooling Temperature (°C) shows a weak screened association with number of sensors with full detachment; largest mean contrast: 15 to 12 to 15 (1.667) vs 15 (1.556).</t>
+          <t>Cooling Temperature (°C) shows a weak screened association with number of sensors with full detachment; largest mean contrast: 15 (1.444) vs 15 to 12 to 15 (1.333).</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
@@ -16706,7 +16631,7 @@
         <v>3</v>
       </c>
       <c r="G51" t="n">
-        <v>0.6491228070175437</v>
+        <v>0.612121212121212</v>
       </c>
       <c r="H51" t="inlineStr">
         <is>
@@ -16715,12 +16640,12 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>Marcos (3.667) vs MOAN (1.667)</t>
+          <t>Marcos (3.667) vs MOAN (2)</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>Trials shows a large screened association with primary Rx2Tx2 change-point count; largest mean contrast: Marcos (3.667) vs MOAN (1.667).</t>
+          <t>Trials shows a large screened association with primary Rx2Tx2 change-point count; largest mean contrast: Marcos (3.667) vs MOAN (2).</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
@@ -16757,7 +16682,7 @@
         <v>2</v>
       </c>
       <c r="G52" t="n">
-        <v>0.4848484848484848</v>
+        <v>0.4838709677419353</v>
       </c>
       <c r="H52" t="inlineStr">
         <is>
@@ -16766,12 +16691,12 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>Marcos Cooling Tunnel (3.667) vs Cooling S (1.889)</t>
+          <t>Marcos Cooling Tunnel (3.667) vs Cooling S (2)</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>Cooling Configuration shows a large screened association with primary Rx2Tx2 change-point count; largest mean contrast: Marcos Cooling Tunnel (3.667) vs Cooling S (1.889).</t>
+          <t>Cooling Configuration shows a large screened association with primary Rx2Tx2 change-point count; largest mean contrast: Marcos Cooling Tunnel (3.667) vs Cooling S (2).</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
@@ -16808,7 +16733,7 @@
         <v>2</v>
       </c>
       <c r="G53" t="n">
-        <v>0.4848484848484848</v>
+        <v>0.4838709677419353</v>
       </c>
       <c r="H53" t="inlineStr">
         <is>
@@ -16817,12 +16742,12 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>15 to 12 to 15 (3.667) vs 15 (1.889)</t>
+          <t>15 to 12 to 15 (3.667) vs 15 (2)</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>Cooling Temperature (°C) shows a large screened association with primary Rx2Tx2 change-point count; largest mean contrast: 15 to 12 to 15 (3.667) vs 15 (1.889).</t>
+          <t>Cooling Temperature (°C) shows a large screened association with primary Rx2Tx2 change-point count; largest mean contrast: 15 to 12 to 15 (3.667) vs 15 (2).</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
@@ -16859,7 +16784,7 @@
         <v>2</v>
       </c>
       <c r="G54" t="n">
-        <v>0.4608294930875576</v>
+        <v>0.4285714285714286</v>
       </c>
       <c r="H54" t="inlineStr">
         <is>
@@ -16868,12 +16793,12 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>20.0 (3) vs 35.0 (1.571)</t>
+          <t>20.0 (3) vs 35.0 (1.714)</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>Cooling Speed (%) shows a large screened association with primary Rx2Tx2 change-point count; largest mean contrast: 20.0 (3) vs 35.0 (1.571).</t>
+          <t>Cooling Speed (%) shows a large screened association with primary Rx2Tx2 change-point count; largest mean contrast: 20.0 (3) vs 35.0 (1.714).</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
@@ -16910,21 +16835,21 @@
         <v>2</v>
       </c>
       <c r="G55" t="n">
-        <v>0.284090909090909</v>
+        <v>0.3903225806451612</v>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>moderate</t>
+          <t>large</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>Dark (2.75) vs Milk (1.5)</t>
+          <t>Dark (2.875) vs Milk (1.5)</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>Chocolate Recipe shows a moderate screened association with primary Rx2Tx2 change-point count; largest mean contrast: Dark (2.75) vs Milk (1.5).</t>
+          <t>Chocolate Recipe shows a large screened association with primary Rx2Tx2 change-point count; largest mean contrast: Dark (2.875) vs Milk (1.5).</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
@@ -16961,21 +16886,21 @@
         <v>2</v>
       </c>
       <c r="G56" t="n">
-        <v>0.284090909090909</v>
+        <v>0.3903225806451612</v>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>moderate</t>
+          <t>large</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>Stella (2.75) vs AMC (1.5)</t>
+          <t>Stella (2.875) vs AMC (1.5)</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>Tempering shows a moderate screened association with primary Rx2Tx2 change-point count; largest mean contrast: Stella (2.75) vs AMC (1.5).</t>
+          <t>Tempering shows a large screened association with primary Rx2Tx2 change-point count; largest mean contrast: Stella (2.875) vs AMC (1.5).</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
@@ -17012,21 +16937,21 @@
         <v>2</v>
       </c>
       <c r="G57" t="n">
-        <v>0.284090909090909</v>
+        <v>0.3903225806451612</v>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>moderate</t>
+          <t>large</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>0.2-0.4 UT (2.75) vs 4.9 (1.5)</t>
+          <t>0.2-0.4 UT (2.875) vs 4.9 (1.5)</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>Tempering Degree shows a moderate screened association with primary Rx2Tx2 change-point count; largest mean contrast: 0.2-0.4 UT (2.75) vs 4.9 (1.5).</t>
+          <t>Tempering Degree shows a large screened association with primary Rx2Tx2 change-point count; largest mean contrast: 0.2-0.4 UT (2.875) vs 4.9 (1.5).</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
@@ -17057,13 +16982,13 @@
         </is>
       </c>
       <c r="E58" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F58" t="n">
         <v>3</v>
       </c>
       <c r="G58" t="n">
-        <v>0.7750684809411131</v>
+        <v>0.733115176184031</v>
       </c>
       <c r="H58" t="inlineStr">
         <is>
@@ -17072,12 +16997,12 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>Marcos (462) vs MOAN (270)</t>
+          <t>Marcos (514) vs HASS (301.5)</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>Trials shows a large screened association with primary Rx2Tx2 detachment duration; largest mean contrast: Marcos (462) vs MOAN (270).</t>
+          <t>Trials shows a large screened association with primary Rx2Tx2 detachment duration; largest mean contrast: Marcos (514) vs HASS (301.5).</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
@@ -17104,17 +17029,17 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Cooling Configuration</t>
+          <t>Chocolate Recipe</t>
         </is>
       </c>
       <c r="E59" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F59" t="n">
         <v>2</v>
       </c>
       <c r="G59" t="n">
-        <v>0.5368831484708115</v>
+        <v>0.5232099084803775</v>
       </c>
       <c r="H59" t="inlineStr">
         <is>
@@ -17123,12 +17048,12 @@
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>Marcos Cooling Tunnel (462) vs Cooling S (225.5)</t>
+          <t>Dark (341.2) vs Milk (154.2)</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>Cooling Configuration shows a large screened association with primary Rx2Tx2 detachment duration; largest mean contrast: Marcos Cooling Tunnel (462) vs Cooling S (225.5).</t>
+          <t>Chocolate Recipe shows a large screened association with primary Rx2Tx2 detachment duration; largest mean contrast: Dark (341.2) vs Milk (154.2).</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
@@ -17155,17 +17080,17 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Cooling Temperature (°C)</t>
+          <t>Tempering</t>
         </is>
       </c>
       <c r="E60" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F60" t="n">
         <v>2</v>
       </c>
       <c r="G60" t="n">
-        <v>0.5368831484708115</v>
+        <v>0.5232099084803775</v>
       </c>
       <c r="H60" t="inlineStr">
         <is>
@@ -17174,12 +17099,12 @@
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>15 to 12 to 15 (462) vs 15 (225.5)</t>
+          <t>Stella (341.2) vs AMC (154.2)</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>Cooling Temperature (°C) shows a large screened association with primary Rx2Tx2 detachment duration; largest mean contrast: 15 to 12 to 15 (462) vs 15 (225.5).</t>
+          <t>Tempering shows a large screened association with primary Rx2Tx2 detachment duration; largest mean contrast: Stella (341.2) vs AMC (154.2).</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
@@ -17206,17 +17131,17 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Chocolate Recipe</t>
+          <t>Tempering Degree</t>
         </is>
       </c>
       <c r="E61" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F61" t="n">
         <v>2</v>
       </c>
       <c r="G61" t="n">
-        <v>0.4819934221539969</v>
+        <v>0.5232099084803775</v>
       </c>
       <c r="H61" t="inlineStr">
         <is>
@@ -17225,12 +17150,12 @@
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>Dark (333.9) vs Milk (154.2)</t>
+          <t>0.2-0.4 UT (341.2) vs 4.9 (154.2)</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>Chocolate Recipe shows a large screened association with primary Rx2Tx2 detachment duration; largest mean contrast: Dark (333.9) vs Milk (154.2).</t>
+          <t>Tempering Degree shows a large screened association with primary Rx2Tx2 detachment duration; largest mean contrast: 0.2-0.4 UT (341.2) vs 4.9 (154.2).</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
@@ -17257,17 +17182,17 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Tempering</t>
+          <t>Cooling Configuration</t>
         </is>
       </c>
       <c r="E62" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F62" t="n">
         <v>2</v>
       </c>
       <c r="G62" t="n">
-        <v>0.4819934221539969</v>
+        <v>0.4249497844018145</v>
       </c>
       <c r="H62" t="inlineStr">
         <is>
@@ -17276,12 +17201,12 @@
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>Stella (333.9) vs AMC (154.2)</t>
+          <t>Marcos Cooling Tunnel (514) vs Cooling S (238.9)</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>Tempering shows a large screened association with primary Rx2Tx2 detachment duration; largest mean contrast: Stella (333.9) vs AMC (154.2).</t>
+          <t>Cooling Configuration shows a large screened association with primary Rx2Tx2 detachment duration; largest mean contrast: Marcos Cooling Tunnel (514) vs Cooling S (238.9).</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
@@ -17308,17 +17233,17 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Tempering Degree</t>
+          <t>Cooling Temperature (°C)</t>
         </is>
       </c>
       <c r="E63" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F63" t="n">
         <v>2</v>
       </c>
       <c r="G63" t="n">
-        <v>0.4819934221539969</v>
+        <v>0.4249497844018145</v>
       </c>
       <c r="H63" t="inlineStr">
         <is>
@@ -17327,12 +17252,12 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>0.2-0.4 UT (333.9) vs 4.9 (154.2)</t>
+          <t>15 to 12 to 15 (514) vs 15 (238.9)</t>
         </is>
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>Tempering Degree shows a large screened association with primary Rx2Tx2 detachment duration; largest mean contrast: 0.2-0.4 UT (333.9) vs 4.9 (154.2).</t>
+          <t>Cooling Temperature (°C) shows a large screened association with primary Rx2Tx2 detachment duration; largest mean contrast: 15 to 12 to 15 (514) vs 15 (238.9).</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
@@ -17369,21 +17294,21 @@
         <v>2</v>
       </c>
       <c r="G64" t="n">
-        <v>0.2017474565239897</v>
+        <v>0.1093561675530039</v>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>moderate</t>
+          <t>small</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>20.0 (301.5) vs 35.0 (203.8)</t>
+          <t>20.0 (301.5) vs 35.0 (221)</t>
         </is>
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>Cooling Speed (%) shows a moderate screened association with primary Rx2Tx2 detachment duration; largest mean contrast: 20.0 (301.5) vs 35.0 (203.8).</t>
+          <t>Cooling Speed (%) shows a small screened association with primary Rx2Tx2 detachment duration; largest mean contrast: 20.0 (301.5) vs 35.0 (221).</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
@@ -17420,21 +17345,21 @@
         <v>2</v>
       </c>
       <c r="G65" t="n">
-        <v>0.2727272727272728</v>
+        <v>0.6</v>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>moderate</t>
+          <t>large</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>Cooling S (1) vs Marcos Cooling Tunnel (0.6667)</t>
+          <t>Cooling S (1) vs Marcos Cooling Tunnel (0.3333)</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>Cooling Configuration shows a moderate screened association with primary Rx2Tx2 full-offset probability; largest mean contrast: Cooling S (1) vs Marcos Cooling Tunnel (0.6667).</t>
+          <t>Cooling Configuration shows a large screened association with primary Rx2Tx2 full-offset probability; largest mean contrast: Cooling S (1) vs Marcos Cooling Tunnel (0.3333).</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
@@ -17471,21 +17396,21 @@
         <v>2</v>
       </c>
       <c r="G66" t="n">
-        <v>0.2727272727272728</v>
+        <v>0.6</v>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>moderate</t>
+          <t>large</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>15 (1) vs 15 to 12 to 15 (0.6667)</t>
+          <t>15 (1) vs 15 to 12 to 15 (0.3333)</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>Cooling Temperature (°C) shows a moderate screened association with primary Rx2Tx2 full-offset probability; largest mean contrast: 15 (1) vs 15 to 12 to 15 (0.6667).</t>
+          <t>Cooling Temperature (°C) shows a large screened association with primary Rx2Tx2 full-offset probability; largest mean contrast: 15 (1) vs 15 to 12 to 15 (0.3333).</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
@@ -17522,21 +17447,21 @@
         <v>3</v>
       </c>
       <c r="G67" t="n">
-        <v>0.2380952380952381</v>
+        <v>0.5555555555555556</v>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>moderate</t>
+          <t>large</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>MOAN (1) vs Marcos (0.6667)</t>
+          <t>MOAN (1) vs Marcos (0.3333)</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>Trials shows a moderate screened association with primary Rx2Tx2 full-offset probability; largest mean contrast: MOAN (1) vs Marcos (0.6667).</t>
+          <t>Trials shows a large screened association with primary Rx2Tx2 full-offset probability; largest mean contrast: MOAN (1) vs Marcos (0.3333).</t>
         </is>
       </c>
       <c r="K67" t="inlineStr">
@@ -17573,21 +17498,21 @@
         <v>2</v>
       </c>
       <c r="G68" t="n">
-        <v>0.04545454545454547</v>
+        <v>0.1</v>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>weak</t>
+          <t>small</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>Milk (1) vs Dark (0.875)</t>
+          <t>Milk (1) vs Dark (0.75)</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>Chocolate Recipe shows a weak screened association with primary Rx2Tx2 full-offset probability; largest mean contrast: Milk (1) vs Dark (0.875).</t>
+          <t>Chocolate Recipe shows a small screened association with primary Rx2Tx2 full-offset probability; largest mean contrast: Milk (1) vs Dark (0.75).</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
@@ -17624,21 +17549,21 @@
         <v>2</v>
       </c>
       <c r="G69" t="n">
-        <v>0.04545454545454547</v>
+        <v>0.1</v>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>weak</t>
+          <t>small</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>AMC (1) vs Stella (0.875)</t>
+          <t>AMC (1) vs Stella (0.75)</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>Tempering shows a weak screened association with primary Rx2Tx2 full-offset probability; largest mean contrast: AMC (1) vs Stella (0.875).</t>
+          <t>Tempering shows a small screened association with primary Rx2Tx2 full-offset probability; largest mean contrast: AMC (1) vs Stella (0.75).</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
@@ -17675,21 +17600,21 @@
         <v>2</v>
       </c>
       <c r="G70" t="n">
-        <v>0.04545454545454547</v>
+        <v>0.1</v>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>weak</t>
+          <t>small</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>4.9 (1) vs 0.2-0.4 UT (0.875)</t>
+          <t>4.9 (1) vs 0.2-0.4 UT (0.75)</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>Tempering Degree shows a weak screened association with primary Rx2Tx2 full-offset probability; largest mean contrast: 4.9 (1) vs 0.2-0.4 UT (0.875).</t>
+          <t>Tempering Degree shows a small screened association with primary Rx2Tx2 full-offset probability; largest mean contrast: 4.9 (1) vs 0.2-0.4 UT (0.75).</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
@@ -18094,11 +18019,11 @@
         <v>1</v>
       </c>
       <c r="I7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Rx1Tx1, Rx2Tx2</t>
+          <t>Rx1Tx1</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -18339,11 +18264,11 @@
         <v>1</v>
       </c>
       <c r="I12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Rx1Tx1, Rx2Tx2</t>
+          <t>Rx2Tx2</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -18788,16 +18713,16 @@
         <v>1</v>
       </c>
       <c r="H5" t="n">
-        <v>250.0007348060608</v>
+        <v>370.000344991684</v>
       </c>
       <c r="I5" t="n">
-        <v>1880.000734806061</v>
+        <v>2000.000344991684</v>
       </c>
       <c r="J5" t="n">
-        <v>595.0007348060608</v>
+        <v>715.000344991684</v>
       </c>
       <c r="K5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L5" t="n">
         <v>2</v>
@@ -18959,11 +18884,11 @@
         <v>2</v>
       </c>
       <c r="L8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>Rx1Tx1, Rx2Tx2</t>
+          <t>Rx1Tx1</t>
         </is>
       </c>
     </row>
@@ -18990,33 +18915,24 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>full_detachment_for_channel</t>
+          <t>partial_detachment_no_change_point_met_threshold</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G9" t="n">
         <v>1</v>
       </c>
-      <c r="H9" t="n">
-        <v>410.0023336410522</v>
-      </c>
-      <c r="I9" t="n">
-        <v>1005.002333641052</v>
-      </c>
-      <c r="J9" t="n">
-        <v>795.0023336410522</v>
-      </c>
       <c r="K9" t="n">
         <v>4</v>
       </c>
       <c r="L9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>Rx1Tx1, Rx2Tx2</t>
+          <t>Rx1Tx1</t>
         </is>
       </c>
     </row>
@@ -19440,33 +19356,24 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>full_detachment_for_channel</t>
+          <t>partial_detachment_no_change_point_met_threshold</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G18" t="n">
         <v>1</v>
       </c>
-      <c r="H18" t="n">
-        <v>413.9799451828003</v>
-      </c>
-      <c r="I18" t="n">
-        <v>1413.9799451828</v>
-      </c>
-      <c r="J18" t="n">
-        <v>1251.9799451828</v>
-      </c>
       <c r="K18" t="n">
         <v>2</v>
       </c>
       <c r="L18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>Rx1Tx1, Rx2Tx2</t>
+          <t>Rx2Tx2</t>
         </is>
       </c>
     </row>
@@ -19515,11 +19422,11 @@
         <v>1</v>
       </c>
       <c r="L19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>Rx1Tx1, Rx2Tx2</t>
+          <t>Rx2Tx2</t>
         </is>
       </c>
     </row>

</xml_diff>